<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-09-22 10:32:16)
</commit_message>
<xml_diff>
--- a/Talabalar_Toliq_Royxati.xlsx
+++ b/Talabalar_Toliq_Royxati.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y169"/>
+  <dimension ref="A1:Y170"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18468,6 +18468,60 @@
         </is>
       </c>
       <c r="Y169" t="inlineStr">
+        <is>
+          <t>KUTILMOQDA</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="n">
+        <v>169</v>
+      </c>
+      <c r="B170" t="inlineStr"/>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>Davolash ishi</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>To'lanmagan</t>
+        </is>
+      </c>
+      <c r="E170" t="inlineStr"/>
+      <c r="F170" t="inlineStr">
+        <is>
+          <t>22.09.2026</t>
+        </is>
+      </c>
+      <c r="G170" t="inlineStr"/>
+      <c r="J170" t="inlineStr"/>
+      <c r="K170" t="inlineStr"/>
+      <c r="L170" t="inlineStr"/>
+      <c r="M170" t="inlineStr"/>
+      <c r="O170" t="inlineStr"/>
+      <c r="Q170" t="inlineStr"/>
+      <c r="R170" t="inlineStr">
+        <is>
+          <t>Umumiy o'rta maktab</t>
+        </is>
+      </c>
+      <c r="S170" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="U170" t="inlineStr">
+        <is>
+          <t>TOPILDI</t>
+        </is>
+      </c>
+      <c r="W170" t="inlineStr">
+        <is>
+          <t>26-01</t>
+        </is>
+      </c>
+      <c r="Y170" t="inlineStr">
         <is>
           <t>KUTILMOQDA</t>
         </is>

</xml_diff>

<commit_message>
Clean phantom row 170, disable vercel cache, and add empty student guard
</commit_message>
<xml_diff>
--- a/Talabalar_Toliq_Royxati.xlsx
+++ b/Talabalar_Toliq_Royxati.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y170"/>
+  <dimension ref="A1:Y169"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18468,60 +18468,6 @@
         </is>
       </c>
       <c r="Y169" t="inlineStr">
-        <is>
-          <t>KUTILMOQDA</t>
-        </is>
-      </c>
-    </row>
-    <row r="170">
-      <c r="A170" t="n">
-        <v>169</v>
-      </c>
-      <c r="B170" t="inlineStr"/>
-      <c r="C170" t="inlineStr">
-        <is>
-          <t>Davolash ishi</t>
-        </is>
-      </c>
-      <c r="D170" t="inlineStr">
-        <is>
-          <t>To'lanmagan</t>
-        </is>
-      </c>
-      <c r="E170" t="inlineStr"/>
-      <c r="F170" t="inlineStr">
-        <is>
-          <t>22.09.2026</t>
-        </is>
-      </c>
-      <c r="G170" t="inlineStr"/>
-      <c r="J170" t="inlineStr"/>
-      <c r="K170" t="inlineStr"/>
-      <c r="L170" t="inlineStr"/>
-      <c r="M170" t="inlineStr"/>
-      <c r="O170" t="inlineStr"/>
-      <c r="Q170" t="inlineStr"/>
-      <c r="R170" t="inlineStr">
-        <is>
-          <t>Umumiy o'rta maktab</t>
-        </is>
-      </c>
-      <c r="S170" t="inlineStr">
-        <is>
-          <t>2024</t>
-        </is>
-      </c>
-      <c r="U170" t="inlineStr">
-        <is>
-          <t>TOPILDI</t>
-        </is>
-      </c>
-      <c r="W170" t="inlineStr">
-        <is>
-          <t>26-01</t>
-        </is>
-      </c>
-      <c r="Y170" t="inlineStr">
         <is>
           <t>KUTILMOQDA</t>
         </is>

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-09-22 10:58:08)
</commit_message>
<xml_diff>
--- a/Talabalar_Toliq_Royxati.xlsx
+++ b/Talabalar_Toliq_Royxati.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y169"/>
+  <dimension ref="A1:Y170"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18468,6 +18468,104 @@
         </is>
       </c>
       <c r="Y169" t="inlineStr">
+        <is>
+          <t>KUTILMOQDA</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="n">
+        <v>169</v>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>Alimova Sevinch</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi - 3 yillik</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>312</t>
+        </is>
+      </c>
+      <c r="F170" t="inlineStr">
+        <is>
+          <t>22.09.2026</t>
+        </is>
+      </c>
+      <c r="G170" t="inlineStr">
+        <is>
+          <t>Raxmiddin qizi</t>
+        </is>
+      </c>
+      <c r="H170" t="inlineStr">
+        <is>
+          <t>Alimova Sevinch Raxmiddin qizi</t>
+        </is>
+      </c>
+      <c r="J170" t="inlineStr">
+        <is>
+          <t>AB7974700</t>
+        </is>
+      </c>
+      <c r="K170" t="inlineStr">
+        <is>
+          <t>62707005740020</t>
+        </is>
+      </c>
+      <c r="L170" t="inlineStr">
+        <is>
+          <t>27.10.2017</t>
+        </is>
+      </c>
+      <c r="M170" t="inlineStr">
+        <is>
+          <t>27.07.2000</t>
+        </is>
+      </c>
+      <c r="N170" t="inlineStr">
+        <is>
+          <t>Mavjud</t>
+        </is>
+      </c>
+      <c r="O170" t="inlineStr"/>
+      <c r="P170" t="inlineStr"/>
+      <c r="Q170" t="inlineStr"/>
+      <c r="R170" t="inlineStr">
+        <is>
+          <t>Shahodatnoma</t>
+        </is>
+      </c>
+      <c r="S170" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="T170" t="inlineStr">
+        <is>
+          <t>700343131</t>
+        </is>
+      </c>
+      <c r="U170" t="inlineStr">
+        <is>
+          <t>TOPILDI</t>
+        </is>
+      </c>
+      <c r="W170" t="inlineStr">
+        <is>
+          <t>26-02</t>
+        </is>
+      </c>
+      <c r="Y170" t="inlineStr">
         <is>
           <t>KUTILMOQDA</t>
         </is>

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-09-22 12:00:22)
</commit_message>
<xml_diff>
--- a/Talabalar_Toliq_Royxati.xlsx
+++ b/Talabalar_Toliq_Royxati.xlsx
@@ -1057,7 +1057,7 @@
       </c>
       <c r="W6" t="inlineStr">
         <is>
-          <t>26-01</t>
+          <t>N</t>
         </is>
       </c>
       <c r="X6" t="inlineStr">
@@ -18537,9 +18537,6 @@
           <t>Mavjud</t>
         </is>
       </c>
-      <c r="O170" t="inlineStr"/>
-      <c r="P170" t="inlineStr"/>
-      <c r="Q170" t="inlineStr"/>
       <c r="R170" t="inlineStr">
         <is>
           <t>Shahodatnoma</t>

</xml_diff>

<commit_message>
feat: Barcha PDF tugmasi endi 7 ta tab emas, 1 ta 7 varaqli yagona A4 PDF (har bir guruh alohida varoqda) qilib ochadi
</commit_message>
<xml_diff>
--- a/Talabalar_Toliq_Royxati.xlsx
+++ b/Talabalar_Toliq_Royxati.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y170"/>
+  <dimension ref="A1:Y171"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18565,6 +18565,66 @@
       <c r="Y170" t="inlineStr">
         <is>
           <t>KUTILMOQDA</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="n">
+        <v>170</v>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>Abdijalolova Dilnura</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi - 3 yillik</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
+      <c r="E171" t="inlineStr"/>
+      <c r="F171" t="inlineStr"/>
+      <c r="G171" t="inlineStr">
+        <is>
+          <t>Yusufjon qizi</t>
+        </is>
+      </c>
+      <c r="H171" t="inlineStr">
+        <is>
+          <t>Abdijalolova Dilnura Yusufjon qizi</t>
+        </is>
+      </c>
+      <c r="J171" t="inlineStr"/>
+      <c r="K171" t="inlineStr"/>
+      <c r="L171" t="inlineStr"/>
+      <c r="M171" t="inlineStr"/>
+      <c r="N171" t="inlineStr">
+        <is>
+          <t>Yo'q</t>
+        </is>
+      </c>
+      <c r="O171" t="inlineStr"/>
+      <c r="P171" t="inlineStr"/>
+      <c r="Q171" t="inlineStr"/>
+      <c r="R171" t="inlineStr">
+        <is>
+          <t>Shahodatnoma</t>
+        </is>
+      </c>
+      <c r="S171" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="T171" t="inlineStr"/>
+      <c r="W171" t="inlineStr">
+        <is>
+          <t>26-01</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-09-22 13:43:56)
</commit_message>
<xml_diff>
--- a/Talabalar_Toliq_Royxati.xlsx
+++ b/Talabalar_Toliq_Royxati.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y171"/>
+  <dimension ref="A1:Y170"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18565,66 +18565,6 @@
       <c r="Y170" t="inlineStr">
         <is>
           <t>KUTILMOQDA</t>
-        </is>
-      </c>
-    </row>
-    <row r="171">
-      <c r="A171" t="n">
-        <v>170</v>
-      </c>
-      <c r="B171" t="inlineStr">
-        <is>
-          <t>Abdijalolova Dilnura</t>
-        </is>
-      </c>
-      <c r="C171" t="inlineStr">
-        <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
-        </is>
-      </c>
-      <c r="D171" t="inlineStr">
-        <is>
-          <t>To'lov qildi</t>
-        </is>
-      </c>
-      <c r="E171" t="inlineStr"/>
-      <c r="F171" t="inlineStr"/>
-      <c r="G171" t="inlineStr">
-        <is>
-          <t>Yusufjon qizi</t>
-        </is>
-      </c>
-      <c r="H171" t="inlineStr">
-        <is>
-          <t>Abdijalolova Dilnura Yusufjon qizi</t>
-        </is>
-      </c>
-      <c r="J171" t="inlineStr"/>
-      <c r="K171" t="inlineStr"/>
-      <c r="L171" t="inlineStr"/>
-      <c r="M171" t="inlineStr"/>
-      <c r="N171" t="inlineStr">
-        <is>
-          <t>Yo'q</t>
-        </is>
-      </c>
-      <c r="O171" t="inlineStr"/>
-      <c r="P171" t="inlineStr"/>
-      <c r="Q171" t="inlineStr"/>
-      <c r="R171" t="inlineStr">
-        <is>
-          <t>Shahodatnoma</t>
-        </is>
-      </c>
-      <c r="S171" t="inlineStr">
-        <is>
-          <t>2024</t>
-        </is>
-      </c>
-      <c r="T171" t="inlineStr"/>
-      <c r="W171" t="inlineStr">
-        <is>
-          <t>26-01</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-09-22 13:45:15)
</commit_message>
<xml_diff>
--- a/Talabalar_Toliq_Royxati.xlsx
+++ b/Talabalar_Toliq_Royxati.xlsx
@@ -5300,6 +5300,11 @@
           <t>Abdijalolova Dilnura</t>
         </is>
       </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi</t>
+        </is>
+      </c>
       <c r="E46" t="inlineStr">
         <is>
           <t>303</t>
@@ -5363,8 +5368,10 @@
           <t>Shahodatnoma</t>
         </is>
       </c>
-      <c r="S46" t="n">
-        <v>2026</v>
+      <c r="S46" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
       </c>
       <c r="T46" t="inlineStr">
         <is>
@@ -5378,7 +5385,7 @@
       </c>
       <c r="W46" t="inlineStr">
         <is>
-          <t>26-03</t>
+          <t>26-01</t>
         </is>
       </c>
       <c r="X46" t="inlineStr">

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-09-22 14:55:29)
</commit_message>
<xml_diff>
--- a/Talabalar_Toliq_Royxati.xlsx
+++ b/Talabalar_Toliq_Royxati.xlsx
@@ -17927,6 +17927,11 @@
           <t>Nazarova Munisa</t>
         </is>
       </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi</t>
+        </is>
+      </c>
       <c r="E164" t="inlineStr">
         <is>
           <t>258</t>
@@ -17972,6 +17977,7 @@
           <t>12.05.1992</t>
         </is>
       </c>
+      <c r="S164" t="inlineStr"/>
       <c r="T164" t="inlineStr">
         <is>
           <t>91-957-18-58</t>
@@ -17984,7 +17990,7 @@
       </c>
       <c r="W164" t="inlineStr">
         <is>
-          <t>26-07</t>
+          <t>26-05</t>
         </is>
       </c>
       <c r="X164" t="inlineStr">

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-09-22 15:05:49)
</commit_message>
<xml_diff>
--- a/Talabalar_Toliq_Royxati.xlsx
+++ b/Talabalar_Toliq_Royxati.xlsx
@@ -16317,14 +16317,14 @@
       </c>
       <c r="H149" t="inlineStr">
         <is>
+          <t>Nurillayeva Sevinch Mashrab qizi</t>
+        </is>
+      </c>
+      <c r="I149" t="inlineStr">
+        <is>
           <t>Nuraliyeva Sevinch Mirsharaf qizi</t>
         </is>
       </c>
-      <c r="I149" t="inlineStr">
-        <is>
-          <t>Nuraliyeva Sevinch Mirsharaf qizi</t>
-        </is>
-      </c>
       <c r="J149" t="inlineStr">
         <is>
           <t>AD9494409</t>
@@ -16347,7 +16347,7 @@
       </c>
       <c r="N149" t="inlineStr">
         <is>
-          <t>Nuraliyeva Sevinch Mirsharaf qizi</t>
+          <t>Mavjud</t>
         </is>
       </c>
       <c r="O149" t="inlineStr">
@@ -16362,7 +16362,7 @@
       </c>
       <c r="Q149" t="inlineStr">
         <is>
-          <t>46-sonli umumiy o'rta ta'lim maktabi</t>
+          <t>46-sonli umumiy o'rta ta'lim maktabini</t>
         </is>
       </c>
       <c r="R149" t="inlineStr">

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-09-22 15:06:50)
</commit_message>
<xml_diff>
--- a/Talabalar_Toliq_Royxati.xlsx
+++ b/Talabalar_Toliq_Royxati.xlsx
@@ -16292,7 +16292,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>Nuraliyeva Sevinch</t>
+          <t>Nurillayeva Sevinch</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
@@ -16312,7 +16312,7 @@
       </c>
       <c r="G149" t="inlineStr">
         <is>
-          <t>Mirsharaf qizi</t>
+          <t>Mashrab qizi</t>
         </is>
       </c>
       <c r="H149" t="inlineStr">

</xml_diff>

<commit_message>
Fix: talabaga fayl biriktirilganda rasmlarni o'z papkasiga ajratish, qulflash va JSHSHIR seriyadek ko'rsatilishi
</commit_message>
<xml_diff>
--- a/Talabalar_Toliq_Royxati.xlsx
+++ b/Talabalar_Toliq_Royxati.xlsx
@@ -16292,7 +16292,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>Nurillayeva Sevinch</t>
+          <t>Nuraliyeva Sevinch</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
@@ -16312,12 +16312,12 @@
       </c>
       <c r="G149" t="inlineStr">
         <is>
-          <t>Mashrab qizi</t>
+          <t>Mirsharaf qizi</t>
         </is>
       </c>
       <c r="H149" t="inlineStr">
         <is>
-          <t>Nurillayeva Sevinch Mashrab qizi</t>
+          <t>Nuraliyeva Sevinch Mirsharaf qizi</t>
         </is>
       </c>
       <c r="I149" t="inlineStr">
@@ -16327,32 +16327,32 @@
       </c>
       <c r="J149" t="inlineStr">
         <is>
-          <t>AD9494409</t>
+          <t>AE4360739</t>
         </is>
       </c>
       <c r="K149" t="inlineStr">
         <is>
-          <t>60504085680019</t>
+          <t>63006085730022</t>
         </is>
       </c>
       <c r="L149" t="inlineStr">
         <is>
-          <t>20.11.2024</t>
+          <t>26.09.2025</t>
         </is>
       </c>
       <c r="M149" t="inlineStr">
         <is>
-          <t>05.04.2008</t>
+          <t>30.06.2008</t>
         </is>
       </c>
       <c r="N149" t="inlineStr">
         <is>
-          <t>Mavjud</t>
+          <t>Nuraliyeva Sevinch Mirsharaf qizi</t>
         </is>
       </c>
       <c r="O149" t="inlineStr">
         <is>
-          <t>UM 03729348</t>
+          <t>UM 03756167</t>
         </is>
       </c>
       <c r="P149" t="inlineStr">
@@ -16362,7 +16362,7 @@
       </c>
       <c r="Q149" t="inlineStr">
         <is>
-          <t>46-sonli umumiy o'rta ta'lim maktabini</t>
+          <t>7-sonli umumiy o'rta ta'lim maktabi</t>
         </is>
       </c>
       <c r="R149" t="inlineStr">
@@ -16370,9 +16370,12 @@
           <t>Shahodatnoma</t>
         </is>
       </c>
-      <c r="S149" t="inlineStr">
-        <is>
-          <t>2026</t>
+      <c r="S149" t="n">
+        <v>2026</v>
+      </c>
+      <c r="T149" t="inlineStr">
+        <is>
+          <t>77-068-30-17</t>
         </is>
       </c>
       <c r="U149" t="inlineStr">

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-09-22 15:32:53)
</commit_message>
<xml_diff>
--- a/Talabalar_Toliq_Royxati.xlsx
+++ b/Talabalar_Toliq_Royxati.xlsx
@@ -16292,7 +16292,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>Nuraliyeva Sevinch</t>
+          <t>Nurillayeva Sevinch</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
@@ -16312,27 +16312,27 @@
       </c>
       <c r="G149" t="inlineStr">
         <is>
-          <t>Mirsharaf qizi</t>
+          <t>Mashrab qizi</t>
         </is>
       </c>
       <c r="H149" t="inlineStr">
         <is>
+          <t>Nurillayeva Sevinch Mashrab qizi</t>
+        </is>
+      </c>
+      <c r="I149" t="inlineStr">
+        <is>
           <t>Nuraliyeva Sevinch Mirsharaf qizi</t>
         </is>
       </c>
-      <c r="I149" t="inlineStr">
-        <is>
-          <t>Nuraliyeva Sevinch Mirsharaf qizi</t>
-        </is>
-      </c>
       <c r="J149" t="inlineStr">
         <is>
-          <t>AE4360739</t>
+          <t>AD9494409</t>
         </is>
       </c>
       <c r="K149" t="inlineStr">
         <is>
-          <t>63006085730022</t>
+          <t>60504085680019</t>
         </is>
       </c>
       <c r="L149" t="inlineStr">
@@ -16342,17 +16342,17 @@
       </c>
       <c r="M149" t="inlineStr">
         <is>
-          <t>30.06.2008</t>
+          <t>05.04.2008</t>
         </is>
       </c>
       <c r="N149" t="inlineStr">
         <is>
-          <t>Nuraliyeva Sevinch Mirsharaf qizi</t>
+          <t>Mavjud</t>
         </is>
       </c>
       <c r="O149" t="inlineStr">
         <is>
-          <t>UM 03756167</t>
+          <t>UM 03729348</t>
         </is>
       </c>
       <c r="P149" t="inlineStr">
@@ -16362,7 +16362,7 @@
       </c>
       <c r="Q149" t="inlineStr">
         <is>
-          <t>7-sonli umumiy o'rta ta'lim maktabi</t>
+          <t>46-sonli umumiy o'rta ta'lim maktabini</t>
         </is>
       </c>
       <c r="R149" t="inlineStr">

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-09-22 15:33:05)
</commit_message>
<xml_diff>
--- a/Talabalar_Toliq_Royxati.xlsx
+++ b/Talabalar_Toliq_Royxati.xlsx
@@ -16370,8 +16370,10 @@
           <t>Shahodatnoma</t>
         </is>
       </c>
-      <c r="S149" t="n">
-        <v>2026</v>
+      <c r="S149" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
       </c>
       <c r="T149" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Rename N-group to Talabalar safidan chiqarilganlar as dedicated special group outside contingent
</commit_message>
<xml_diff>
--- a/Talabalar_Toliq_Royxati.xlsx
+++ b/Talabalar_Toliq_Royxati.xlsx
@@ -852,7 +852,7 @@
       </c>
       <c r="W4" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Talabalar safidan chiqarilganlar</t>
         </is>
       </c>
       <c r="X4" t="inlineStr">
@@ -1057,7 +1057,7 @@
       </c>
       <c r="W6" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Talabalar safidan chiqarilganlar</t>
         </is>
       </c>
       <c r="X6" t="inlineStr">

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-09-22 21:02:23)
</commit_message>
<xml_diff>
--- a/Talabalar_Toliq_Royxati.xlsx
+++ b/Talabalar_Toliq_Royxati.xlsx
@@ -10117,14 +10117,10 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Qodirova Shabnam</t>
-        </is>
-      </c>
-      <c r="C91" t="inlineStr">
-        <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
-        </is>
-      </c>
+          <t>Qodirova Sabina</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr"/>
       <c r="E91" t="inlineStr">
         <is>
           <t>137</t>
@@ -10137,7 +10133,7 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>O'tkir qizi</t>
+          <t>Suxrob qizi</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
@@ -10150,54 +10146,28 @@
           <t>Qodirova Shabnam O'tkir qizi</t>
         </is>
       </c>
-      <c r="J91" t="inlineStr">
-        <is>
-          <t>AE5242435</t>
-        </is>
-      </c>
-      <c r="K91" t="inlineStr">
-        <is>
-          <t>61807085680045</t>
-        </is>
-      </c>
-      <c r="L91" t="inlineStr">
-        <is>
-          <t>01.12.2025</t>
-        </is>
-      </c>
-      <c r="M91" t="inlineStr">
-        <is>
-          <t>18.07.2008</t>
-        </is>
-      </c>
+      <c r="J91" t="inlineStr"/>
+      <c r="K91" t="inlineStr"/>
+      <c r="L91" t="inlineStr"/>
+      <c r="M91" t="inlineStr"/>
       <c r="N91" t="inlineStr">
         <is>
           <t>Qodirova Shabnam O'tkir qizi</t>
         </is>
       </c>
-      <c r="O91" t="inlineStr">
-        <is>
-          <t>UM 03729278</t>
-        </is>
-      </c>
+      <c r="O91" t="inlineStr"/>
       <c r="P91" t="inlineStr">
         <is>
           <t>https://e-shahodatnoma.uz/api/public/getcertpdf/3934766/3452539/98763bcf-ef33-4ddb-b3e1-ddf8c7990688?preview=true</t>
         </is>
       </c>
-      <c r="Q91" t="inlineStr">
-        <is>
-          <t>44-sonli umumiy o'rta ta'lim maktabi</t>
-        </is>
-      </c>
+      <c r="Q91" t="inlineStr"/>
       <c r="R91" t="inlineStr">
         <is>
           <t>Shahodatnoma</t>
         </is>
       </c>
-      <c r="S91" t="n">
-        <v>2026</v>
-      </c>
+      <c r="S91" t="inlineStr"/>
       <c r="T91" t="inlineStr">
         <is>
           <t>88-827-07-18, 88-386-04-85</t>

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-09-22 21:08:04)
</commit_message>
<xml_diff>
--- a/Talabalar_Toliq_Royxati.xlsx
+++ b/Talabalar_Toliq_Royxati.xlsx
@@ -10120,7 +10120,11 @@
           <t>Qodirova Sabina</t>
         </is>
       </c>
-      <c r="C91" t="inlineStr"/>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi</t>
+        </is>
+      </c>
       <c r="E91" t="inlineStr">
         <is>
           <t>137</t>
@@ -10138,7 +10142,7 @@
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>Qodirova Shabnam O'tkir qizi</t>
+          <t>Qodirova Sabina Suxrob qizi</t>
         </is>
       </c>
       <c r="I91" t="inlineStr">

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-09-22 21:20:19)
</commit_message>
<xml_diff>
--- a/Talabalar_Toliq_Royxati.xlsx
+++ b/Talabalar_Toliq_Royxati.xlsx
@@ -10165,7 +10165,11 @@
           <t>https://e-shahodatnoma.uz/api/public/getcertpdf/3934766/3452539/98763bcf-ef33-4ddb-b3e1-ddf8c7990688?preview=true</t>
         </is>
       </c>
-      <c r="Q91" t="inlineStr"/>
+      <c r="Q91" t="inlineStr">
+        <is>
+          <t>TEST-SINOV-123</t>
+        </is>
+      </c>
       <c r="R91" t="inlineStr">
         <is>
           <t>Shahodatnoma</t>

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-09-22 21:22:17)
</commit_message>
<xml_diff>
--- a/Talabalar_Toliq_Royxati.xlsx
+++ b/Talabalar_Toliq_Royxati.xlsx
@@ -10165,11 +10165,7 @@
           <t>https://e-shahodatnoma.uz/api/public/getcertpdf/3934766/3452539/98763bcf-ef33-4ddb-b3e1-ddf8c7990688?preview=true</t>
         </is>
       </c>
-      <c r="Q91" t="inlineStr">
-        <is>
-          <t>TEST-SINOV-123</t>
-        </is>
-      </c>
+      <c r="Q91" t="inlineStr"/>
       <c r="R91" t="inlineStr">
         <is>
           <t>Shahodatnoma</t>

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-09-22 21:37:50)
</commit_message>
<xml_diff>
--- a/Talabalar_Toliq_Royxati.xlsx
+++ b/Talabalar_Toliq_Royxati.xlsx
@@ -10150,28 +10150,26 @@
           <t>Qodirova Shabnam O'tkir qizi</t>
         </is>
       </c>
-      <c r="J91" t="inlineStr"/>
-      <c r="K91" t="inlineStr"/>
-      <c r="L91" t="inlineStr"/>
-      <c r="M91" t="inlineStr"/>
       <c r="N91" t="inlineStr">
         <is>
           <t>Qodirova Shabnam O'tkir qizi</t>
         </is>
       </c>
-      <c r="O91" t="inlineStr"/>
       <c r="P91" t="inlineStr">
         <is>
           <t>https://e-shahodatnoma.uz/api/public/getcertpdf/3934766/3452539/98763bcf-ef33-4ddb-b3e1-ddf8c7990688?preview=true</t>
         </is>
       </c>
-      <c r="Q91" t="inlineStr"/>
+      <c r="Q91" t="inlineStr">
+        <is>
+          <t>OLCHOV-1</t>
+        </is>
+      </c>
       <c r="R91" t="inlineStr">
         <is>
           <t>Shahodatnoma</t>
         </is>
       </c>
-      <c r="S91" t="inlineStr"/>
       <c r="T91" t="inlineStr">
         <is>
           <t>88-827-07-18, 88-386-04-85</t>

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-09-22 21:45:07)
</commit_message>
<xml_diff>
--- a/Talabalar_Toliq_Royxati.xlsx
+++ b/Talabalar_Toliq_Royxati.xlsx
@@ -10160,11 +10160,7 @@
           <t>https://e-shahodatnoma.uz/api/public/getcertpdf/3934766/3452539/98763bcf-ef33-4ddb-b3e1-ddf8c7990688?preview=true</t>
         </is>
       </c>
-      <c r="Q91" t="inlineStr">
-        <is>
-          <t>BATCH-C</t>
-        </is>
-      </c>
+      <c r="Q91" t="inlineStr"/>
       <c r="R91" t="inlineStr">
         <is>
           <t>Shahodatnoma</t>

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-09-22 21:46:26)
</commit_message>
<xml_diff>
--- a/Talabalar_Toliq_Royxati.xlsx
+++ b/Talabalar_Toliq_Royxati.xlsx
@@ -10150,11 +10150,16 @@
           <t>Qodirova Shabnam O'tkir qizi</t>
         </is>
       </c>
+      <c r="J91" t="inlineStr"/>
+      <c r="K91" t="inlineStr"/>
+      <c r="L91" t="inlineStr"/>
+      <c r="M91" t="inlineStr"/>
       <c r="N91" t="inlineStr">
         <is>
           <t>Qodirova Shabnam O'tkir qizi</t>
         </is>
       </c>
+      <c r="O91" t="inlineStr"/>
       <c r="P91" t="inlineStr">
         <is>
           <t>https://e-shahodatnoma.uz/api/public/getcertpdf/3934766/3452539/98763bcf-ef33-4ddb-b3e1-ddf8c7990688?preview=true</t>
@@ -10166,6 +10171,7 @@
           <t>Shahodatnoma</t>
         </is>
       </c>
+      <c r="S91" t="inlineStr"/>
       <c r="T91" t="inlineStr">
         <is>
           <t>88-827-07-18, 88-386-04-85</t>

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-09-22 22:10:52)
</commit_message>
<xml_diff>
--- a/Talabalar_Toliq_Royxati.xlsx
+++ b/Talabalar_Toliq_Royxati.xlsx
@@ -10150,28 +10150,26 @@
           <t>Qodirova Shabnam O'tkir qizi</t>
         </is>
       </c>
-      <c r="J91" t="inlineStr"/>
-      <c r="K91" t="inlineStr"/>
-      <c r="L91" t="inlineStr"/>
-      <c r="M91" t="inlineStr"/>
       <c r="N91" t="inlineStr">
         <is>
           <t>Qodirova Shabnam O'tkir qizi</t>
         </is>
       </c>
-      <c r="O91" t="inlineStr"/>
       <c r="P91" t="inlineStr">
         <is>
           <t>https://e-shahodatnoma.uz/api/public/getcertpdf/3934766/3452539/98763bcf-ef33-4ddb-b3e1-ddf8c7990688?preview=true</t>
         </is>
       </c>
-      <c r="Q91" t="inlineStr"/>
+      <c r="Q91" t="inlineStr">
+        <is>
+          <t>OLCHOV-2</t>
+        </is>
+      </c>
       <c r="R91" t="inlineStr">
         <is>
           <t>Shahodatnoma</t>
         </is>
       </c>
-      <c r="S91" t="inlineStr"/>
       <c r="T91" t="inlineStr">
         <is>
           <t>88-827-07-18, 88-386-04-85</t>

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-09-22 22:11:39)
</commit_message>
<xml_diff>
--- a/Talabalar_Toliq_Royxati.xlsx
+++ b/Talabalar_Toliq_Royxati.xlsx
@@ -10160,11 +10160,7 @@
           <t>https://e-shahodatnoma.uz/api/public/getcertpdf/3934766/3452539/98763bcf-ef33-4ddb-b3e1-ddf8c7990688?preview=true</t>
         </is>
       </c>
-      <c r="Q91" t="inlineStr">
-        <is>
-          <t>OLCHOV-2</t>
-        </is>
-      </c>
+      <c r="Q91" t="inlineStr"/>
       <c r="R91" t="inlineStr">
         <is>
           <t>Shahodatnoma</t>

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-09-22 22:19:13)
</commit_message>
<xml_diff>
--- a/Talabalar_Toliq_Royxati.xlsx
+++ b/Talabalar_Toliq_Royxati.xlsx
@@ -10117,7 +10117,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Qodirova Sabina</t>
+          <t>Qodirova Sabinaa</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
@@ -10142,7 +10142,7 @@
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>Qodirova Sabina Suxrob qizi</t>
+          <t>Qodirova Sabinaa Suxrob qizi</t>
         </is>
       </c>
       <c r="I91" t="inlineStr">
@@ -10150,11 +10150,20 @@
           <t>Qodirova Shabnam O'tkir qizi</t>
         </is>
       </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>AB</t>
+        </is>
+      </c>
+      <c r="K91" t="inlineStr"/>
+      <c r="L91" t="inlineStr"/>
+      <c r="M91" t="inlineStr"/>
       <c r="N91" t="inlineStr">
         <is>
           <t>Qodirova Shabnam O'tkir qizi</t>
         </is>
       </c>
+      <c r="O91" t="inlineStr"/>
       <c r="P91" t="inlineStr">
         <is>
           <t>https://e-shahodatnoma.uz/api/public/getcertpdf/3934766/3452539/98763bcf-ef33-4ddb-b3e1-ddf8c7990688?preview=true</t>
@@ -10166,6 +10175,7 @@
           <t>Shahodatnoma</t>
         </is>
       </c>
+      <c r="S91" t="inlineStr"/>
       <c r="T91" t="inlineStr">
         <is>
           <t>88-827-07-18, 88-386-04-85</t>

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-09-22 22:28:05)
</commit_message>
<xml_diff>
--- a/Talabalar_Toliq_Royxati.xlsx
+++ b/Talabalar_Toliq_Royxati.xlsx
@@ -10169,7 +10169,11 @@
           <t>https://e-shahodatnoma.uz/api/public/getcertpdf/3934766/3452539/98763bcf-ef33-4ddb-b3e1-ddf8c7990688?preview=true</t>
         </is>
       </c>
-      <c r="Q91" t="inlineStr"/>
+      <c r="Q91" t="inlineStr">
+        <is>
+          <t>TUGMA-SINOV</t>
+        </is>
+      </c>
       <c r="R91" t="inlineStr">
         <is>
           <t>Shahodatnoma</t>

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-09-22 22:29:16)
</commit_message>
<xml_diff>
--- a/Talabalar_Toliq_Royxati.xlsx
+++ b/Talabalar_Toliq_Royxati.xlsx
@@ -10169,11 +10169,7 @@
           <t>https://e-shahodatnoma.uz/api/public/getcertpdf/3934766/3452539/98763bcf-ef33-4ddb-b3e1-ddf8c7990688?preview=true</t>
         </is>
       </c>
-      <c r="Q91" t="inlineStr">
-        <is>
-          <t>TUGMA-SINOV</t>
-        </is>
-      </c>
+      <c r="Q91" t="inlineStr"/>
       <c r="R91" t="inlineStr">
         <is>
           <t>Shahodatnoma</t>

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-09-22 22:33:01)
</commit_message>
<xml_diff>
--- a/Talabalar_Toliq_Royxati.xlsx
+++ b/Talabalar_Toliq_Royxati.xlsx
@@ -10117,7 +10117,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Qodirova Sabinaa</t>
+          <t>Qodirova Sabina</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
@@ -10142,7 +10142,7 @@
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>Qodirova Sabinaa Suxrob qizi</t>
+          <t>Qodirova Sabina Suxrob qizi</t>
         </is>
       </c>
       <c r="I91" t="inlineStr">
@@ -10150,11 +10150,7 @@
           <t>Qodirova Shabnam O'tkir qizi</t>
         </is>
       </c>
-      <c r="J91" t="inlineStr">
-        <is>
-          <t>AB</t>
-        </is>
-      </c>
+      <c r="J91" t="inlineStr"/>
       <c r="K91" t="inlineStr"/>
       <c r="L91" t="inlineStr"/>
       <c r="M91" t="inlineStr"/>

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-09-23 09:47:35)
</commit_message>
<xml_diff>
--- a/Talabalar_Toliq_Royxati.xlsx
+++ b/Talabalar_Toliq_Royxati.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y170"/>
+  <dimension ref="A1:Y171"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10150,28 +10150,21 @@
           <t>Qodirova Shabnam O'tkir qizi</t>
         </is>
       </c>
-      <c r="J91" t="inlineStr"/>
-      <c r="K91" t="inlineStr"/>
-      <c r="L91" t="inlineStr"/>
-      <c r="M91" t="inlineStr"/>
       <c r="N91" t="inlineStr">
         <is>
           <t>Qodirova Shabnam O'tkir qizi</t>
         </is>
       </c>
-      <c r="O91" t="inlineStr"/>
       <c r="P91" t="inlineStr">
         <is>
           <t>https://e-shahodatnoma.uz/api/public/getcertpdf/3934766/3452539/98763bcf-ef33-4ddb-b3e1-ddf8c7990688?preview=true</t>
         </is>
       </c>
-      <c r="Q91" t="inlineStr"/>
       <c r="R91" t="inlineStr">
         <is>
           <t>Shahodatnoma</t>
         </is>
       </c>
-      <c r="S91" t="inlineStr"/>
       <c r="T91" t="inlineStr">
         <is>
           <t>88-827-07-18, 88-386-04-85</t>
@@ -18564,6 +18557,94 @@
       <c r="Y170" t="inlineStr">
         <is>
           <t>TASDIQLANDI</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="n">
+        <v>170</v>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>Mahmatqulova Nilufar</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi - 3 yillik</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>314</t>
+        </is>
+      </c>
+      <c r="F171" t="inlineStr"/>
+      <c r="G171" t="inlineStr">
+        <is>
+          <t>Qayum qizi</t>
+        </is>
+      </c>
+      <c r="H171" t="inlineStr">
+        <is>
+          <t>Mahmatqulova Nilufar Qayum qizi</t>
+        </is>
+      </c>
+      <c r="J171" t="inlineStr">
+        <is>
+          <t>AE6047826</t>
+        </is>
+      </c>
+      <c r="K171" t="inlineStr">
+        <is>
+          <t>60806085590115</t>
+        </is>
+      </c>
+      <c r="L171" t="inlineStr">
+        <is>
+          <t>26.01.2026</t>
+        </is>
+      </c>
+      <c r="M171" t="inlineStr">
+        <is>
+          <t>08.06.2008</t>
+        </is>
+      </c>
+      <c r="N171" t="inlineStr">
+        <is>
+          <t>Mavjud</t>
+        </is>
+      </c>
+      <c r="O171" t="inlineStr">
+        <is>
+          <t>UM 03754788</t>
+        </is>
+      </c>
+      <c r="P171" t="inlineStr"/>
+      <c r="Q171" t="inlineStr">
+        <is>
+          <t>43-sonli umumiy o'rta ta'lim maktabini</t>
+        </is>
+      </c>
+      <c r="R171" t="inlineStr">
+        <is>
+          <t>Shahodatnoma</t>
+        </is>
+      </c>
+      <c r="S171" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="T171" t="inlineStr"/>
+      <c r="W171" t="inlineStr">
+        <is>
+          <t>26-06</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-09-23 09:48:18)
</commit_message>
<xml_diff>
--- a/Talabalar_Toliq_Royxati.xlsx
+++ b/Talabalar_Toliq_Royxati.xlsx
@@ -18584,7 +18584,6 @@
           <t>314</t>
         </is>
       </c>
-      <c r="F171" t="inlineStr"/>
       <c r="G171" t="inlineStr">
         <is>
           <t>Qayum qizi</t>
@@ -18625,7 +18624,6 @@
           <t>UM 03754788</t>
         </is>
       </c>
-      <c r="P171" t="inlineStr"/>
       <c r="Q171" t="inlineStr">
         <is>
           <t>43-sonli umumiy o'rta ta'lim maktabini</t>
@@ -18641,10 +18639,14 @@
           <t>2024</t>
         </is>
       </c>
-      <c r="T171" t="inlineStr"/>
       <c r="W171" t="inlineStr">
         <is>
           <t>26-06</t>
+        </is>
+      </c>
+      <c r="Y171" t="inlineStr">
+        <is>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-09-23 13:32:01)
</commit_message>
<xml_diff>
--- a/Talabalar_Toliq_Royxati.xlsx
+++ b/Talabalar_Toliq_Royxati.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y171"/>
+  <dimension ref="A1:Y172"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17569,7 +17569,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>G‘aniyeva Asila</t>
+          <t>G'aniyeva Asila</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
@@ -17587,44 +17587,44 @@
       </c>
       <c r="G161" t="inlineStr">
         <is>
-          <t>G‘ani qizi</t>
+          <t>G'ani qizi</t>
         </is>
       </c>
       <c r="H161" t="inlineStr">
         <is>
+          <t>G'aniyeva Asila G'ani qizi</t>
+        </is>
+      </c>
+      <c r="I161" t="inlineStr">
+        <is>
           <t>G‘aniyeva Asila G‘ani qizi</t>
         </is>
       </c>
-      <c r="I161" t="inlineStr">
+      <c r="J161" t="inlineStr">
+        <is>
+          <t>AE5575300</t>
+        </is>
+      </c>
+      <c r="K161" t="inlineStr">
+        <is>
+          <t>41011925590038</t>
+        </is>
+      </c>
+      <c r="L161" t="inlineStr">
+        <is>
+          <t>23.12.2025</t>
+        </is>
+      </c>
+      <c r="M161" t="inlineStr">
+        <is>
+          <t>10.11.1992</t>
+        </is>
+      </c>
+      <c r="N161" t="inlineStr">
         <is>
           <t>G‘aniyeva Asila G‘ani qizi</t>
         </is>
       </c>
-      <c r="J161" t="inlineStr">
-        <is>
-          <t>AE5575300</t>
-        </is>
-      </c>
-      <c r="K161" t="inlineStr">
-        <is>
-          <t>41011925590038</t>
-        </is>
-      </c>
-      <c r="L161" t="inlineStr">
-        <is>
-          <t>23.12.2025</t>
-        </is>
-      </c>
-      <c r="M161" t="inlineStr">
-        <is>
-          <t>10.11.1992</t>
-        </is>
-      </c>
-      <c r="N161" t="inlineStr">
-        <is>
-          <t>G‘aniyeva Asila G‘ani qizi</t>
-        </is>
-      </c>
       <c r="O161" t="inlineStr">
         <is>
           <t>L 125287</t>
@@ -17657,7 +17657,7 @@
       </c>
       <c r="W161" t="inlineStr">
         <is>
-          <t>26-07</t>
+          <t>26-04</t>
         </is>
       </c>
       <c r="X161" t="inlineStr">
@@ -18647,6 +18647,91 @@
       <c r="Y171" t="inlineStr">
         <is>
           <t>TASDIQLANDI</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="n">
+        <v>171</v>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>Izzatulloyeva Vazira</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi - 3 yillik</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>383</t>
+        </is>
+      </c>
+      <c r="G172" t="inlineStr">
+        <is>
+          <t>G'ayratzoda</t>
+        </is>
+      </c>
+      <c r="H172" t="inlineStr">
+        <is>
+          <t>Izzatulloyeva Vazira G'ayratzoda</t>
+        </is>
+      </c>
+      <c r="J172" t="inlineStr">
+        <is>
+          <t>AE5671026</t>
+        </is>
+      </c>
+      <c r="K172" t="inlineStr">
+        <is>
+          <t>42004975680094</t>
+        </is>
+      </c>
+      <c r="L172" t="inlineStr">
+        <is>
+          <t>05.01.2026</t>
+        </is>
+      </c>
+      <c r="M172" t="inlineStr">
+        <is>
+          <t>20.04.1997</t>
+        </is>
+      </c>
+      <c r="N172" t="inlineStr">
+        <is>
+          <t>Mavjud</t>
+        </is>
+      </c>
+      <c r="O172" t="inlineStr">
+        <is>
+          <t>K 4174595</t>
+        </is>
+      </c>
+      <c r="Q172" t="inlineStr">
+        <is>
+          <t>Kitob agrobiznes kasb-hunar kolleji</t>
+        </is>
+      </c>
+      <c r="R172" t="inlineStr">
+        <is>
+          <t>Diplom</t>
+        </is>
+      </c>
+      <c r="S172" t="inlineStr">
+        <is>
+          <t>2016</t>
+        </is>
+      </c>
+      <c r="W172" t="inlineStr">
+        <is>
+          <t>26-03</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-09-23 13:33:51)
</commit_message>
<xml_diff>
--- a/Talabalar_Toliq_Royxati.xlsx
+++ b/Talabalar_Toliq_Royxati.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y172"/>
+  <dimension ref="A1:Y173"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18732,6 +18732,94 @@
       <c r="W172" t="inlineStr">
         <is>
           <t>26-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="n">
+        <v>172</v>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>Xujamuratova Durdona</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi - 3 yillik</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>232</t>
+        </is>
+      </c>
+      <c r="F173" t="inlineStr"/>
+      <c r="G173" t="inlineStr">
+        <is>
+          <t>Bahrom qizi</t>
+        </is>
+      </c>
+      <c r="H173" t="inlineStr">
+        <is>
+          <t>Xujamuratova Durdona Bahrom qizi</t>
+        </is>
+      </c>
+      <c r="J173" t="inlineStr">
+        <is>
+          <t>AE5954513</t>
+        </is>
+      </c>
+      <c r="K173" t="inlineStr">
+        <is>
+          <t>62204085720105</t>
+        </is>
+      </c>
+      <c r="L173" t="inlineStr">
+        <is>
+          <t>20.01.2026</t>
+        </is>
+      </c>
+      <c r="M173" t="inlineStr">
+        <is>
+          <t>22.04.2008</t>
+        </is>
+      </c>
+      <c r="N173" t="inlineStr">
+        <is>
+          <t>Mavjud</t>
+        </is>
+      </c>
+      <c r="O173" t="inlineStr">
+        <is>
+          <t>UM 03717652</t>
+        </is>
+      </c>
+      <c r="P173" t="inlineStr"/>
+      <c r="Q173" t="inlineStr">
+        <is>
+          <t>19-sonli umumiy o'rta ta'lim maktabini</t>
+        </is>
+      </c>
+      <c r="R173" t="inlineStr">
+        <is>
+          <t>Shahodatnoma</t>
+        </is>
+      </c>
+      <c r="S173" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="T173" t="inlineStr"/>
+      <c r="W173" t="inlineStr">
+        <is>
+          <t>26-04</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-09-23 13:35:12)
</commit_message>
<xml_diff>
--- a/Talabalar_Toliq_Royxati.xlsx
+++ b/Talabalar_Toliq_Royxati.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y173"/>
+  <dimension ref="A1:Y174"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18759,7 +18759,6 @@
           <t>232</t>
         </is>
       </c>
-      <c r="F173" t="inlineStr"/>
       <c r="G173" t="inlineStr">
         <is>
           <t>Bahrom qizi</t>
@@ -18800,7 +18799,6 @@
           <t>UM 03717652</t>
         </is>
       </c>
-      <c r="P173" t="inlineStr"/>
       <c r="Q173" t="inlineStr">
         <is>
           <t>19-sonli umumiy o'rta ta'lim maktabini</t>
@@ -18816,8 +18814,95 @@
           <t>2024</t>
         </is>
       </c>
-      <c r="T173" t="inlineStr"/>
       <c r="W173" t="inlineStr">
+        <is>
+          <t>26-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="n">
+        <v>173</v>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>Ulugbekova Zara</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi - 3 yillik</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>313</t>
+        </is>
+      </c>
+      <c r="F174" t="inlineStr"/>
+      <c r="G174" t="inlineStr">
+        <is>
+          <t>Ulug'bek qizi</t>
+        </is>
+      </c>
+      <c r="H174" t="inlineStr">
+        <is>
+          <t>Ulugbekova Zara Ulug'bek qizi</t>
+        </is>
+      </c>
+      <c r="J174" t="inlineStr">
+        <is>
+          <t>AE4760779</t>
+        </is>
+      </c>
+      <c r="K174" t="inlineStr">
+        <is>
+          <t>61109085590127</t>
+        </is>
+      </c>
+      <c r="L174" t="inlineStr">
+        <is>
+          <t>24.10.2025</t>
+        </is>
+      </c>
+      <c r="M174" t="inlineStr">
+        <is>
+          <t>11.09.2008</t>
+        </is>
+      </c>
+      <c r="N174" t="inlineStr">
+        <is>
+          <t>Mavjud</t>
+        </is>
+      </c>
+      <c r="O174" t="inlineStr">
+        <is>
+          <t>UM 03728161</t>
+        </is>
+      </c>
+      <c r="P174" t="inlineStr"/>
+      <c r="Q174" t="inlineStr">
+        <is>
+          <t>5-sonli umumiy o'rta ta'lim maktabini</t>
+        </is>
+      </c>
+      <c r="R174" t="inlineStr">
+        <is>
+          <t>Shahodatnoma</t>
+        </is>
+      </c>
+      <c r="S174" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="T174" t="inlineStr"/>
+      <c r="W174" t="inlineStr">
         <is>
           <t>26-04</t>
         </is>

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-09-23 16:28:06)
</commit_message>
<xml_diff>
--- a/Talabalar_Toliq_Royxati.xlsx
+++ b/Talabalar_Toliq_Royxati.xlsx
@@ -11602,21 +11602,44 @@
           <t>Qodirova Shabnam O'tkir qizi</t>
         </is>
       </c>
+      <c r="J106" t="inlineStr">
+        <is>
+          <t>AC2359638</t>
+        </is>
+      </c>
+      <c r="K106" t="inlineStr">
+        <is>
+          <t>602030 4568 0015</t>
+        </is>
+      </c>
+      <c r="L106" t="inlineStr">
+        <is>
+          <t>03.11.2019</t>
+        </is>
+      </c>
+      <c r="M106" t="inlineStr">
+        <is>
+          <t>02.03.2004</t>
+        </is>
+      </c>
       <c r="N106" t="inlineStr">
         <is>
           <t>Qodirova Shabnam O'tkir qizi</t>
         </is>
       </c>
+      <c r="O106" t="inlineStr"/>
       <c r="P106" t="inlineStr">
         <is>
           <t>https://e-shahodatnoma.uz/api/public/getcertpdf/3934766/3452539/98763bcf-ef33-4ddb-b3e1-ddf8c7990688?preview=true</t>
         </is>
       </c>
+      <c r="Q106" t="inlineStr"/>
       <c r="R106" t="inlineStr">
         <is>
           <t>Shahodatnoma</t>
         </is>
       </c>
+      <c r="S106" t="inlineStr"/>
       <c r="T106" t="inlineStr">
         <is>
           <t>88-827-07-18, 88-386-04-85</t>

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-09-23 16:32:03)
</commit_message>
<xml_diff>
--- a/Talabalar_Toliq_Royxati.xlsx
+++ b/Talabalar_Toliq_Royxati.xlsx
@@ -11627,19 +11627,16 @@
           <t>Qodirova Shabnam O'tkir qizi</t>
         </is>
       </c>
-      <c r="O106" t="inlineStr"/>
       <c r="P106" t="inlineStr">
         <is>
           <t>https://e-shahodatnoma.uz/api/public/getcertpdf/3934766/3452539/98763bcf-ef33-4ddb-b3e1-ddf8c7990688?preview=true</t>
         </is>
       </c>
-      <c r="Q106" t="inlineStr"/>
       <c r="R106" t="inlineStr">
         <is>
           <t>Shahodatnoma</t>
         </is>
       </c>
-      <c r="S106" t="inlineStr"/>
       <c r="T106" t="inlineStr">
         <is>
           <t>88-827-07-18, 88-386-04-85</t>
@@ -17521,7 +17518,7 @@
       </c>
       <c r="Y161" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-09-24 08:50:02)
</commit_message>
<xml_diff>
--- a/Talabalar_Toliq_Royxati.xlsx
+++ b/Talabalar_Toliq_Royxati.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y174"/>
+  <dimension ref="A1:Y175"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18922,6 +18922,94 @@
       <c r="Y174" t="inlineStr">
         <is>
           <t>TASDIQLANDI</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="n">
+        <v>174</v>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>Ixtiyorova Niginabonu</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi - 3 yillik</t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>227</t>
+        </is>
+      </c>
+      <c r="F175" t="inlineStr"/>
+      <c r="G175" t="inlineStr">
+        <is>
+          <t>Xolovna</t>
+        </is>
+      </c>
+      <c r="H175" t="inlineStr">
+        <is>
+          <t>Ixtiyorova Niginabonu Xolovna</t>
+        </is>
+      </c>
+      <c r="J175" t="inlineStr">
+        <is>
+          <t>AD9335686</t>
+        </is>
+      </c>
+      <c r="K175" t="inlineStr">
+        <is>
+          <t>60710085680054</t>
+        </is>
+      </c>
+      <c r="L175" t="inlineStr">
+        <is>
+          <t>09.11.2024</t>
+        </is>
+      </c>
+      <c r="M175" t="inlineStr">
+        <is>
+          <t>07.10.2008</t>
+        </is>
+      </c>
+      <c r="N175" t="inlineStr">
+        <is>
+          <t>Mavjud</t>
+        </is>
+      </c>
+      <c r="O175" t="inlineStr">
+        <is>
+          <t>um 03729467</t>
+        </is>
+      </c>
+      <c r="P175" t="inlineStr"/>
+      <c r="Q175" t="inlineStr">
+        <is>
+          <t>51-maktab</t>
+        </is>
+      </c>
+      <c r="R175" t="inlineStr">
+        <is>
+          <t>Shahodatnoma</t>
+        </is>
+      </c>
+      <c r="S175" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="T175" t="inlineStr"/>
+      <c r="W175" t="inlineStr">
+        <is>
+          <t>26-05</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-09-24 10:36:11)
</commit_message>
<xml_diff>
--- a/Talabalar_Toliq_Royxati.xlsx
+++ b/Talabalar_Toliq_Royxati.xlsx
@@ -9466,7 +9466,7 @@
       </c>
       <c r="R85" t="inlineStr">
         <is>
-          <t>Kasb-hunar kolleji diplomi</t>
+          <t>Shahodatnoma</t>
         </is>
       </c>
       <c r="S85" t="inlineStr">
@@ -9474,6 +9474,7 @@
           <t>2018</t>
         </is>
       </c>
+      <c r="T85" t="inlineStr"/>
       <c r="U85" t="inlineStr">
         <is>
           <t>TOPILDI</t>
@@ -9486,7 +9487,7 @@
       </c>
       <c r="W85" t="inlineStr">
         <is>
-          <t>26-07</t>
+          <t>26-06</t>
         </is>
       </c>
       <c r="X85" t="inlineStr">

</xml_diff>

<commit_message>
Add 5 students to group 26-06 with docx extraction and duplicate Passport/JSHSHIR warning system
</commit_message>
<xml_diff>
--- a/Talabalar_Toliq_Royxati.xlsx
+++ b/Talabalar_Toliq_Royxati.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y174"/>
+  <dimension ref="A1:Y178"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9404,6 +9404,11 @@
           <t>Hamshiralik ishi - 3 yillik</t>
         </is>
       </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E85" t="inlineStr">
         <is>
           <t>212</t>
@@ -9411,7 +9416,7 @@
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>2026-09-02 00:00:00</t>
+          <t>22.08.2026</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
@@ -9461,12 +9466,12 @@
       </c>
       <c r="Q85" t="inlineStr">
         <is>
-          <t>Kitob san'at va xizmat ko'rsatish kasb-hunar kolleji</t>
+          <t>Kitob sanoat va xizmat ko'rsatish kasb-hunar kolleji</t>
         </is>
       </c>
       <c r="R85" t="inlineStr">
         <is>
-          <t>Shahodatnoma</t>
+          <t>Diplom</t>
         </is>
       </c>
       <c r="S85" t="inlineStr">
@@ -9474,10 +9479,9 @@
           <t>2018</t>
         </is>
       </c>
-      <c r="T85" t="inlineStr"/>
       <c r="U85" t="inlineStr">
         <is>
-          <t>TOPILDI</t>
+          <t>To'liq</t>
         </is>
       </c>
       <c r="V85" t="inlineStr">
@@ -18898,6 +18902,261 @@
       <c r="W174" t="inlineStr">
         <is>
           <t>26-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="n">
+        <v>174</v>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>Abdunazarova Dilafro'z</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi - 3 yillik</t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>273</t>
+        </is>
+      </c>
+      <c r="F175" t="inlineStr">
+        <is>
+          <t>07.09.2026</t>
+        </is>
+      </c>
+      <c r="G175" t="inlineStr">
+        <is>
+          <t>Burxon qizi</t>
+        </is>
+      </c>
+      <c r="H175" t="inlineStr">
+        <is>
+          <t>Abdunazarova Dilafro'z Burxon qizi</t>
+        </is>
+      </c>
+      <c r="I175" t="inlineStr">
+        <is>
+          <t>Abdinazarova Dilafro'z Burxon qizi</t>
+        </is>
+      </c>
+      <c r="J175" t="inlineStr">
+        <is>
+          <t>AE3704528</t>
+        </is>
+      </c>
+      <c r="K175" t="inlineStr">
+        <is>
+          <t>40401955680037</t>
+        </is>
+      </c>
+      <c r="L175" t="inlineStr">
+        <is>
+          <t>08.08.2025</t>
+        </is>
+      </c>
+      <c r="M175" t="inlineStr">
+        <is>
+          <t>04.01.1995</t>
+        </is>
+      </c>
+      <c r="N175" t="inlineStr">
+        <is>
+          <t>Abdinazarova Dilafro'z Burxon qizi</t>
+        </is>
+      </c>
+      <c r="O175" t="inlineStr">
+        <is>
+          <t>K 3745934</t>
+        </is>
+      </c>
+      <c r="Q175" t="inlineStr">
+        <is>
+          <t>Kitob iqtisodiyot kolleji</t>
+        </is>
+      </c>
+      <c r="R175" t="inlineStr">
+        <is>
+          <t>Diplom</t>
+        </is>
+      </c>
+      <c r="S175" t="inlineStr">
+        <is>
+          <t>2015</t>
+        </is>
+      </c>
+      <c r="T175" t="inlineStr">
+        <is>
+          <t>90-341-06-76 / 91-898-04-95</t>
+        </is>
+      </c>
+      <c r="U175" t="inlineStr">
+        <is>
+          <t>To'liq</t>
+        </is>
+      </c>
+      <c r="W175" t="inlineStr">
+        <is>
+          <t>26-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="n">
+        <v>175</v>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>Azimova Zaxro</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi - 3 yillik</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
+      <c r="G176" t="inlineStr">
+        <is>
+          <t>Abdirouf qizi</t>
+        </is>
+      </c>
+      <c r="H176" t="inlineStr">
+        <is>
+          <t>Azimova Zaxro Abdirouf qizi</t>
+        </is>
+      </c>
+      <c r="I176" t="inlineStr">
+        <is>
+          <t>Azimova Zaxro Abdirouf qizi</t>
+        </is>
+      </c>
+      <c r="R176" t="inlineStr">
+        <is>
+          <t>Shahodatnoma</t>
+        </is>
+      </c>
+      <c r="U176" t="inlineStr">
+        <is>
+          <t>Chala</t>
+        </is>
+      </c>
+      <c r="W176" t="inlineStr">
+        <is>
+          <t>26-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="n">
+        <v>176</v>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>Uzoqova Fazilat</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi - 3 yillik</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
+      <c r="G177" t="inlineStr">
+        <is>
+          <t>Nurali qizi</t>
+        </is>
+      </c>
+      <c r="H177" t="inlineStr">
+        <is>
+          <t>Uzoqova Fazilat Nurali qizi</t>
+        </is>
+      </c>
+      <c r="I177" t="inlineStr">
+        <is>
+          <t>Uzoqova Fazilat Nurali qizi</t>
+        </is>
+      </c>
+      <c r="R177" t="inlineStr">
+        <is>
+          <t>Shahodatnoma</t>
+        </is>
+      </c>
+      <c r="U177" t="inlineStr">
+        <is>
+          <t>Chala</t>
+        </is>
+      </c>
+      <c r="W177" t="inlineStr">
+        <is>
+          <t>26-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="n">
+        <v>177</v>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>Sayfiyeva Sarvinoz</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi - 3 yillik</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
+      <c r="G178" t="inlineStr">
+        <is>
+          <t>Zafar qizi</t>
+        </is>
+      </c>
+      <c r="H178" t="inlineStr">
+        <is>
+          <t>Sayfiyeva Sarvinoz Zafar qizi</t>
+        </is>
+      </c>
+      <c r="I178" t="inlineStr">
+        <is>
+          <t>Sayfiyeva Sarvinoz Zafar qizi</t>
+        </is>
+      </c>
+      <c r="R178" t="inlineStr">
+        <is>
+          <t>Shahodatnoma</t>
+        </is>
+      </c>
+      <c r="U178" t="inlineStr">
+        <is>
+          <t>Chala</t>
+        </is>
+      </c>
+      <c r="W178" t="inlineStr">
+        <is>
+          <t>26-06</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-09-24 13:55:47)
</commit_message>
<xml_diff>
--- a/Talabalar_Toliq_Royxati.xlsx
+++ b/Talabalar_Toliq_Royxati.xlsx
@@ -19016,7 +19016,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>Azimova Zaxro</t>
+          <t>Azimova Zahroxon</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
@@ -19031,22 +19031,67 @@
       </c>
       <c r="G176" t="inlineStr">
         <is>
-          <t>Abdirouf qizi</t>
+          <t>Abdirauf qizi</t>
         </is>
       </c>
       <c r="H176" t="inlineStr">
         <is>
+          <t>Azimova Zahroxon Abdirauf qizi</t>
+        </is>
+      </c>
+      <c r="I176" t="inlineStr">
+        <is>
           <t>Azimova Zaxro Abdirouf qizi</t>
         </is>
       </c>
-      <c r="I176" t="inlineStr">
-        <is>
-          <t>Azimova Zaxro Abdirouf qizi</t>
+      <c r="J176" t="inlineStr">
+        <is>
+          <t>AD5290004</t>
+        </is>
+      </c>
+      <c r="K176" t="inlineStr">
+        <is>
+          <t>61312065590013</t>
+        </is>
+      </c>
+      <c r="L176" t="inlineStr">
+        <is>
+          <t>01.12.2023</t>
+        </is>
+      </c>
+      <c r="M176" t="inlineStr">
+        <is>
+          <t>13.12.2006</t>
+        </is>
+      </c>
+      <c r="N176" t="inlineStr">
+        <is>
+          <t>Mavjud</t>
+        </is>
+      </c>
+      <c r="O176" t="inlineStr">
+        <is>
+          <t>PT № 0176926</t>
+        </is>
+      </c>
+      <c r="Q176" t="inlineStr">
+        <is>
+          <t>Shahrisabz shahar 2-son kasb-hunar maktabi</t>
         </is>
       </c>
       <c r="R176" t="inlineStr">
         <is>
-          <t>Shahodatnoma</t>
+          <t>Diplom</t>
+        </is>
+      </c>
+      <c r="S176" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="T176" t="inlineStr">
+        <is>
+          <t>977997671</t>
         </is>
       </c>
       <c r="U176" t="inlineStr">

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-09-24 13:57:00)
</commit_message>
<xml_diff>
--- a/Talabalar_Toliq_Royxati.xlsx
+++ b/Talabalar_Toliq_Royxati.xlsx
@@ -19029,6 +19029,11 @@
           <t>To'lov qildi</t>
         </is>
       </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>318</t>
+        </is>
+      </c>
       <c r="G176" t="inlineStr">
         <is>
           <t>Abdirauf qizi</t>
@@ -19102,6 +19107,11 @@
       <c r="W176" t="inlineStr">
         <is>
           <t>26-06</t>
+        </is>
+      </c>
+      <c r="Y176" t="inlineStr">
+        <is>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-09-24 13:59:01)
</commit_message>
<xml_diff>
--- a/Talabalar_Toliq_Royxati.xlsx
+++ b/Talabalar_Toliq_Royxati.xlsx
@@ -19009,6 +19009,11 @@
           <t>26-06</t>
         </is>
       </c>
+      <c r="Y175" t="inlineStr">
+        <is>
+          <t>TASDIQLANDI</t>
+        </is>
+      </c>
     </row>
     <row r="176">
       <c r="A176" t="n">

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-09-24 14:50:33)
</commit_message>
<xml_diff>
--- a/Talabalar_Toliq_Royxati.xlsx
+++ b/Talabalar_Toliq_Royxati.xlsx
@@ -19204,6 +19204,31 @@
           <t>Sayfiyeva Sarvinoz Zafar qizi</t>
         </is>
       </c>
+      <c r="J178" t="inlineStr">
+        <is>
+          <t>AB6304158</t>
+        </is>
+      </c>
+      <c r="K178" t="inlineStr">
+        <is>
+          <t>28071542703279</t>
+        </is>
+      </c>
+      <c r="L178" t="inlineStr">
+        <is>
+          <t>28.03.2017</t>
+        </is>
+      </c>
+      <c r="M178" t="inlineStr">
+        <is>
+          <t>15.07.1998</t>
+        </is>
+      </c>
+      <c r="N178" t="inlineStr">
+        <is>
+          <t>Mavjud</t>
+        </is>
+      </c>
       <c r="R178" t="inlineStr">
         <is>
           <t>Shahodatnoma</t>

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-09-24 14:57:09)
</commit_message>
<xml_diff>
--- a/Talabalar_Toliq_Royxati.xlsx
+++ b/Talabalar_Toliq_Royxati.xlsx
@@ -19211,7 +19211,7 @@
       </c>
       <c r="K178" t="inlineStr">
         <is>
-          <t>41507985590024</t>
+          <t>41507985590074</t>
         </is>
       </c>
       <c r="L178" t="inlineStr">
@@ -19229,9 +19229,24 @@
           <t>Mavjud</t>
         </is>
       </c>
+      <c r="O178" t="inlineStr">
+        <is>
+          <t>K № 4587984</t>
+        </is>
+      </c>
+      <c r="Q178" t="inlineStr">
+        <is>
+          <t>KASBIY KOLLEJ</t>
+        </is>
+      </c>
       <c r="R178" t="inlineStr">
         <is>
-          <t>Shahodatnoma</t>
+          <t>Diplom</t>
+        </is>
+      </c>
+      <c r="S178" t="inlineStr">
+        <is>
+          <t>2018</t>
         </is>
       </c>
       <c r="U178" t="inlineStr">

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-09-24 14:58:28)
</commit_message>
<xml_diff>
--- a/Talabalar_Toliq_Royxati.xlsx
+++ b/Talabalar_Toliq_Royxati.xlsx
@@ -19176,7 +19176,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>Sayfiyeva Sarvinoz</t>
+          <t>Sayfieva Sarvinoz</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
@@ -19189,6 +19189,7 @@
           <t>To'lov qildi</t>
         </is>
       </c>
+      <c r="E178" t="inlineStr"/>
       <c r="G178" t="inlineStr">
         <is>
           <t>Zafar qizi</t>
@@ -19196,14 +19197,14 @@
       </c>
       <c r="H178" t="inlineStr">
         <is>
+          <t>Sayfieva Sarvinoz Zafar qizi</t>
+        </is>
+      </c>
+      <c r="I178" t="inlineStr">
+        <is>
           <t>Sayfiyeva Sarvinoz Zafar qizi</t>
         </is>
       </c>
-      <c r="I178" t="inlineStr">
-        <is>
-          <t>Sayfiyeva Sarvinoz Zafar qizi</t>
-        </is>
-      </c>
       <c r="J178" t="inlineStr">
         <is>
           <t>AB6304158</t>
@@ -19211,7 +19212,7 @@
       </c>
       <c r="K178" t="inlineStr">
         <is>
-          <t>41507985590074</t>
+          <t>415079 8559 0074</t>
         </is>
       </c>
       <c r="L178" t="inlineStr">
@@ -19231,12 +19232,12 @@
       </c>
       <c r="O178" t="inlineStr">
         <is>
-          <t>K № 4587984</t>
+          <t>K 4587984</t>
         </is>
       </c>
       <c r="Q178" t="inlineStr">
         <is>
-          <t>KASBIY KOLLEJ</t>
+          <t>Shahrisabz qurulish va maishiy texnikalar kasb-hunar kolleji</t>
         </is>
       </c>
       <c r="R178" t="inlineStr">
@@ -19249,6 +19250,7 @@
           <t>2018</t>
         </is>
       </c>
+      <c r="T178" t="inlineStr"/>
       <c r="U178" t="inlineStr">
         <is>
           <t>Chala</t>

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-09-24 15:05:22)
</commit_message>
<xml_diff>
--- a/Talabalar_Toliq_Royxati.xlsx
+++ b/Talabalar_Toliq_Royxati.xlsx
@@ -8259,6 +8259,12 @@
           <t>Muminova Durdona</t>
         </is>
       </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr"/>
       <c r="F74" t="inlineStr">
         <is>
           <t>2026-09-17 00:00:00</t>
@@ -8274,6 +8280,19 @@
           <t>Muminova Durdona Anvar qizi</t>
         </is>
       </c>
+      <c r="J74" t="inlineStr"/>
+      <c r="K74" t="inlineStr"/>
+      <c r="L74" t="inlineStr"/>
+      <c r="M74" t="inlineStr"/>
+      <c r="O74" t="inlineStr"/>
+      <c r="Q74" t="inlineStr"/>
+      <c r="R74" t="inlineStr">
+        <is>
+          <t>Shahodatnoma</t>
+        </is>
+      </c>
+      <c r="S74" t="inlineStr"/>
+      <c r="T74" t="inlineStr"/>
       <c r="U74" t="inlineStr">
         <is>
           <t>FAYL_YOQ</t>
@@ -8286,7 +8305,7 @@
       </c>
       <c r="W74" t="inlineStr">
         <is>
-          <t>26-06</t>
+          <t>Talabalar safidan chiqarilganlar</t>
         </is>
       </c>
       <c r="X74" t="inlineStr">
@@ -19189,7 +19208,6 @@
           <t>To'lov qildi</t>
         </is>
       </c>
-      <c r="E178" t="inlineStr"/>
       <c r="G178" t="inlineStr">
         <is>
           <t>Zafar qizi</t>
@@ -19250,7 +19268,6 @@
           <t>2018</t>
         </is>
       </c>
-      <c r="T178" t="inlineStr"/>
       <c r="U178" t="inlineStr">
         <is>
           <t>Chala</t>

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-09-24 15:42:23)
</commit_message>
<xml_diff>
--- a/Talabalar_Toliq_Royxati.xlsx
+++ b/Talabalar_Toliq_Royxati.xlsx
@@ -781,6 +781,11 @@
           <t>Abdixalilova Shohzoda</t>
         </is>
       </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E4" t="inlineStr">
         <is>
           <t>274</t>
@@ -1016,6 +1021,11 @@
           <t>Hamshiralik ishi - 3 yillik</t>
         </is>
       </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E6" t="inlineStr">
         <is>
           <t>140</t>
@@ -1126,6 +1136,11 @@
           <t>Hamshiralik ishi - 3 yillik</t>
         </is>
       </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E7" t="inlineStr">
         <is>
           <t>203</t>
@@ -1236,6 +1251,11 @@
           <t>Feldsherlik ishi</t>
         </is>
       </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E8" t="inlineStr">
         <is>
           <t>204</t>
@@ -1346,6 +1366,11 @@
           <t>Hamshiralik ishi - 3 yillik</t>
         </is>
       </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E9" t="inlineStr">
         <is>
           <t>33</t>
@@ -1651,6 +1676,11 @@
           <t>Farmatsiya ishi</t>
         </is>
       </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E12" t="inlineStr">
         <is>
           <t>182</t>
@@ -1871,6 +1901,11 @@
           <t>Hamshiralik ishi - 3 yillik</t>
         </is>
       </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E14" t="inlineStr">
         <is>
           <t>224</t>
@@ -1981,9 +2016,14 @@
           <t>Hamshiralik ishi</t>
         </is>
       </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>265</t>
+          <t>258</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -2081,6 +2121,11 @@
           <t>Farmatsiya ishi</t>
         </is>
       </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E16" t="inlineStr">
         <is>
           <t>229</t>
@@ -2191,6 +2236,11 @@
           <t>Feldsherlik ishi</t>
         </is>
       </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E17" t="inlineStr">
         <is>
           <t>86</t>
@@ -2301,6 +2351,11 @@
           <t>Hamshiralik ishi - 3 yillik</t>
         </is>
       </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E18" t="inlineStr">
         <is>
           <t>44</t>
@@ -2526,6 +2581,11 @@
           <t>Hamshiralik ishi - 3 yillik</t>
         </is>
       </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E20" t="inlineStr">
         <is>
           <t>239</t>
@@ -2731,6 +2791,11 @@
           <t>Davlatova Gulnoza</t>
         </is>
       </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E22" t="inlineStr">
         <is>
           <t>310</t>
@@ -2952,6 +3017,11 @@
           <t>Farmatsiya ishi</t>
         </is>
       </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E24" t="inlineStr">
         <is>
           <t>45</t>
@@ -3057,6 +3127,11 @@
           <t>Hamshiralik ishi - 3 yillik</t>
         </is>
       </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E25" t="inlineStr">
         <is>
           <t>174</t>
@@ -3157,6 +3232,11 @@
           <t>Hamshiralik ishi - 3 yillik</t>
         </is>
       </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E26" t="inlineStr">
         <is>
           <t>110</t>
@@ -3367,9 +3447,14 @@
           <t>Hamshiralik ishi - 3 yillik</t>
         </is>
       </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>135</t>
+          <t>5</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -3796,6 +3881,11 @@
           <t>Hamshiralik ishi - 3 yillik</t>
         </is>
       </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E32" t="inlineStr">
         <is>
           <t>236</t>
@@ -3906,6 +3996,11 @@
           <t>Hamshiralik ishi - 3 yillik</t>
         </is>
       </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E33" t="inlineStr">
         <is>
           <t>97</t>
@@ -4111,6 +4206,11 @@
           <t>Hamshiralik ishi - 3 yillik</t>
         </is>
       </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E35" t="inlineStr">
         <is>
           <t>26</t>
@@ -4324,6 +4424,11 @@
           <t>Hamroqulova Marjona</t>
         </is>
       </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E37" t="inlineStr">
         <is>
           <t>275</t>
@@ -4444,6 +4549,11 @@
           <t>Hamshiralik ishi - 3 yillik</t>
         </is>
       </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E38" t="inlineStr">
         <is>
           <t>166</t>
@@ -4659,6 +4769,11 @@
           <t>Farmatsiya ishi</t>
         </is>
       </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E40" t="inlineStr">
         <is>
           <t>167</t>
@@ -4879,9 +4994,14 @@
           <t>Hamshiralik ishi - 3 yillik</t>
         </is>
       </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>129</t>
+          <t>292</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -5092,6 +5212,11 @@
           <t>Hamshiralik ishi</t>
         </is>
       </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E44" t="inlineStr">
         <is>
           <t>294</t>
@@ -5197,6 +5322,11 @@
           <t>Hamshiralik ishi - 3 yillik</t>
         </is>
       </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E45" t="inlineStr">
         <is>
           <t>94</t>
@@ -5307,6 +5437,11 @@
           <t>Hamshiralik ishi - 3 yillik</t>
         </is>
       </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E46" t="inlineStr">
         <is>
           <t>65</t>
@@ -5507,6 +5642,11 @@
           <t>Hamshiralik ishi - 3 yillik</t>
         </is>
       </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E48" t="inlineStr">
         <is>
           <t>202</t>
@@ -5617,6 +5757,11 @@
           <t>Hamshiralik ishi - 3 yillik</t>
         </is>
       </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E49" t="inlineStr">
         <is>
           <t>95</t>
@@ -5727,6 +5872,11 @@
           <t>Hamshiralik ishi - 3 yillik</t>
         </is>
       </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E50" t="inlineStr">
         <is>
           <t>17</t>
@@ -5837,6 +5987,11 @@
           <t>Feldsherlik ishi</t>
         </is>
       </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E51" t="inlineStr">
         <is>
           <t>211</t>
@@ -5932,6 +6087,11 @@
           <t>Hamshiralik ishi</t>
         </is>
       </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E52" t="inlineStr">
         <is>
           <t>262</t>
@@ -6042,6 +6202,11 @@
           <t>Hamshiralik ishi - 3 yillik</t>
         </is>
       </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E53" t="inlineStr">
         <is>
           <t>173</t>
@@ -6152,6 +6317,11 @@
           <t>Hamshiralik ishi - 3 yillik</t>
         </is>
       </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E54" t="inlineStr">
         <is>
           <t>18</t>
@@ -6262,9 +6432,14 @@
           <t>Hamshiralik ishi - 2 yillik</t>
         </is>
       </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>59</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -6482,6 +6657,11 @@
           <t>Hamshiralik ishi - 3 yillik</t>
         </is>
       </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E57" t="inlineStr">
         <is>
           <t>215</t>
@@ -6592,6 +6772,11 @@
           <t>Karimova Nozliya</t>
         </is>
       </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E58" t="inlineStr">
         <is>
           <t>250</t>
@@ -6797,6 +6982,11 @@
           <t>Hamshiralik ishi - 3 yillik</t>
         </is>
       </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E60" t="inlineStr">
         <is>
           <t>139</t>
@@ -6907,6 +7097,11 @@
           <t>Hamshiralik ishi - 3 yillik</t>
         </is>
       </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E61" t="inlineStr">
         <is>
           <t>390</t>
@@ -7102,6 +7297,11 @@
           <t>Mahmudova Gulsanam</t>
         </is>
       </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E63" t="inlineStr">
         <is>
           <t>277</t>
@@ -7215,6 +7415,11 @@
           <t>Hamshiralik ishi - 3 yillik</t>
         </is>
       </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E64" t="inlineStr">
         <is>
           <t>120</t>
@@ -7430,6 +7635,11 @@
           <t>Hamshiralik ishi - 3 yillik</t>
         </is>
       </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E66" t="inlineStr">
         <is>
           <t>199</t>
@@ -7535,6 +7745,11 @@
           <t>Mansurova Gulasal</t>
         </is>
       </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E67" t="inlineStr">
         <is>
           <t>301</t>
@@ -7728,6 +7943,11 @@
           <t>Hamshiralik ishi - 3 yillik</t>
         </is>
       </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E69" t="inlineStr">
         <is>
           <t>101</t>
@@ -7838,9 +8058,14 @@
           <t>Hamshiralik ishi - 3 yillik</t>
         </is>
       </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>311</t>
+          <t>11</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
@@ -7956,6 +8181,11 @@
           <t>Hamshiralik ishi - 3 yillik</t>
         </is>
       </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E71" t="inlineStr">
         <is>
           <t>60</t>
@@ -8056,9 +8286,14 @@
           <t>Hamshiralik ishi</t>
         </is>
       </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>281</t>
+          <t>26</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
@@ -8264,7 +8499,6 @@
           <t>Hamshiralik ishi</t>
         </is>
       </c>
-      <c r="E74" t="inlineStr"/>
       <c r="F74" t="inlineStr">
         <is>
           <t>2026-09-17 00:00:00</t>
@@ -8280,19 +8514,11 @@
           <t>Muminova Durdona Anvar qizi</t>
         </is>
       </c>
-      <c r="J74" t="inlineStr"/>
-      <c r="K74" t="inlineStr"/>
-      <c r="L74" t="inlineStr"/>
-      <c r="M74" t="inlineStr"/>
-      <c r="O74" t="inlineStr"/>
-      <c r="Q74" t="inlineStr"/>
       <c r="R74" t="inlineStr">
         <is>
           <t>Shahodatnoma</t>
         </is>
       </c>
-      <c r="S74" t="inlineStr"/>
-      <c r="T74" t="inlineStr"/>
       <c r="U74" t="inlineStr">
         <is>
           <t>FAYL_YOQ</t>
@@ -8333,6 +8559,11 @@
           <t>Hamshiralik ishi - 3 yillik</t>
         </is>
       </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E75" t="inlineStr">
         <is>
           <t>163</t>
@@ -8443,9 +8674,14 @@
           <t>Hamshiralik ishi - 3 yillik</t>
         </is>
       </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>169</t>
+          <t>167</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -8548,6 +8784,11 @@
           <t>Hamshiralik ishi - 3 yillik</t>
         </is>
       </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E77" t="inlineStr">
         <is>
           <t>72</t>
@@ -9097,6 +9338,11 @@
           <t>Hamshiralik ishi - 3 yillik</t>
         </is>
       </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E82" t="inlineStr">
         <is>
           <t>176</t>
@@ -9823,6 +10069,11 @@
           <t>Niyozova Sevara</t>
         </is>
       </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E89" t="inlineStr">
         <is>
           <t>304</t>
@@ -9878,6 +10129,11 @@
           <t>Hamshiralik ishi - 3 yillik</t>
         </is>
       </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E90" t="inlineStr">
         <is>
           <t>231</t>
@@ -10093,6 +10349,11 @@
           <t>Hamshiralik ishi - 3 yillik</t>
         </is>
       </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E92" t="inlineStr">
         <is>
           <t>106</t>
@@ -10203,6 +10464,11 @@
           <t>Hamshiralik ishi - 3 yillik</t>
         </is>
       </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E93" t="inlineStr">
         <is>
           <t>38</t>
@@ -10428,6 +10694,11 @@
           <t>Hamshiralik ishi - 3 yillik</t>
         </is>
       </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E95" t="inlineStr">
         <is>
           <t>87</t>
@@ -10738,6 +11009,11 @@
           <t>Hamshiralik ishi - 3 yillik</t>
         </is>
       </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E98" t="inlineStr">
         <is>
           <t>47</t>
@@ -10951,6 +11227,11 @@
           <t>Hamshiralik ishi - 2 yillik</t>
         </is>
       </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E100" t="inlineStr">
         <is>
           <t>90</t>
@@ -11061,6 +11342,11 @@
           <t>Hamshiralik ishi - 3 yillik</t>
         </is>
       </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E101" t="inlineStr">
         <is>
           <t>105</t>
@@ -11281,6 +11567,11 @@
           <t>Hamshiralik ishi</t>
         </is>
       </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E103" t="inlineStr">
         <is>
           <t>251</t>
@@ -11381,9 +11672,14 @@
           <t>Hamshiralik ishi - 3 yillik</t>
         </is>
       </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>56</t>
+          <t>55</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
@@ -11491,9 +11787,14 @@
           <t>Hamshiralik ishi</t>
         </is>
       </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>137</t>
+          <t>295</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
@@ -11701,6 +12002,11 @@
           <t>Hamshiralik ishi - 3 yillik</t>
         </is>
       </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E107" t="inlineStr">
         <is>
           <t>242</t>
@@ -11816,6 +12122,11 @@
           <t>Hamshiralik ishi - 2 yillik</t>
         </is>
       </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E108" t="inlineStr">
         <is>
           <t>392</t>
@@ -12041,6 +12352,11 @@
           <t>Hamshiralik ishi</t>
         </is>
       </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E110" t="inlineStr">
         <is>
           <t>291</t>
@@ -12529,9 +12845,14 @@
           <t>Hamshiralik ishi - 3 yillik</t>
         </is>
       </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>84</t>
+          <t>81</t>
         </is>
       </c>
       <c r="F115" t="inlineStr">
@@ -12744,6 +13065,11 @@
           <t>Hamshiralik ishi</t>
         </is>
       </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E117" t="inlineStr">
         <is>
           <t>254</t>
@@ -12954,6 +13280,11 @@
           <t>Saydalimova Ruxshona</t>
         </is>
       </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E119" t="inlineStr">
         <is>
           <t>74</t>
@@ -13064,9 +13395,14 @@
           <t>Sayfillayeva Shodiyona</t>
         </is>
       </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>03</t>
+          <t>3</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
@@ -13399,6 +13735,11 @@
           <t>Hamshiralik ishi - 3 yillik</t>
         </is>
       </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E123" t="inlineStr">
         <is>
           <t>107</t>
@@ -13509,6 +13850,11 @@
           <t>Hamshiralik ishi - 3 yillik</t>
         </is>
       </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E124" t="inlineStr">
         <is>
           <t>57</t>
@@ -13619,6 +13965,11 @@
           <t>Hamshiralik ishi - 3 yillik</t>
         </is>
       </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E125" t="inlineStr">
         <is>
           <t>162</t>
@@ -13729,6 +14080,11 @@
           <t>Hamshiralik ishi - 3 yillik</t>
         </is>
       </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E126" t="inlineStr">
         <is>
           <t>172</t>
@@ -13834,6 +14190,11 @@
           <t>Hamshiralik ishi</t>
         </is>
       </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E127" t="inlineStr">
         <is>
           <t>288</t>
@@ -14150,6 +14511,11 @@
           <t>Hamshiralik ishi - 2 yillik</t>
         </is>
       </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E130" t="inlineStr">
         <is>
           <t>20</t>
@@ -14260,6 +14626,11 @@
           <t>Hamshiralik ishi</t>
         </is>
       </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E131" t="inlineStr">
         <is>
           <t>299</t>
@@ -14355,6 +14726,11 @@
           <t>To'raboyeva Sabrina</t>
         </is>
       </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E132" t="inlineStr">
         <is>
           <t>6</t>
@@ -14465,6 +14841,11 @@
           <t>Hamshiralik ishi - 2 yillik</t>
         </is>
       </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E133" t="inlineStr">
         <is>
           <t>11</t>
@@ -14570,6 +14951,11 @@
           <t>Hamshiralik ishi - 3 yillik</t>
         </is>
       </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E134" t="inlineStr">
         <is>
           <t>388</t>
@@ -14675,6 +15061,11 @@
           <t>Hamshiralik ishi - 3 yillik</t>
         </is>
       </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E135" t="inlineStr">
         <is>
           <t>112</t>
@@ -14785,6 +15176,11 @@
           <t>Hamshiralik ishi - 3 yillik</t>
         </is>
       </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E136" t="inlineStr">
         <is>
           <t>161</t>
@@ -14990,6 +15386,11 @@
           <t>Hamshiralik ishi - 2 yillik</t>
         </is>
       </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E138" t="inlineStr">
         <is>
           <t>21</t>
@@ -15100,9 +15501,14 @@
           <t>Farmatsiya ishi</t>
         </is>
       </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>222</t>
+          <t>122</t>
         </is>
       </c>
       <c r="F139" t="inlineStr">
@@ -15310,6 +15716,11 @@
           <t>Tursunova Aziza</t>
         </is>
       </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E141" t="inlineStr">
         <is>
           <t>276</t>
@@ -15838,9 +16249,14 @@
           <t>Hamshiralik ishi - 3 yillik</t>
         </is>
       </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>73</t>
+          <t>79</t>
         </is>
       </c>
       <c r="F146" t="inlineStr">
@@ -16051,6 +16467,11 @@
           <t>Hamshiralik ishi - 3 yillik</t>
         </is>
       </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E148" t="inlineStr">
         <is>
           <t>148</t>
@@ -16166,6 +16587,11 @@
           <t>Hamshiralik ishi</t>
         </is>
       </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E149" t="inlineStr">
         <is>
           <t>279</t>
@@ -16367,6 +16793,11 @@
           <t>Hamshiralik ishi - 3 yillik</t>
         </is>
       </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E151" t="inlineStr">
         <is>
           <t>188</t>
@@ -16587,6 +17018,11 @@
           <t>Hamshiralik ishi - 3 yillik</t>
         </is>
       </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E153" t="inlineStr">
         <is>
           <t>14</t>
@@ -16784,6 +17220,11 @@
           <t>Hamshiralik ishi - 3 yillik</t>
         </is>
       </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E155" t="inlineStr">
         <is>
           <t>113</t>
@@ -16894,6 +17335,11 @@
           <t>Hamshiralik ishi - 3 yillik</t>
         </is>
       </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E156" t="inlineStr">
         <is>
           <t>116</t>
@@ -16999,6 +17445,11 @@
           <t>Hamshiralik ishi - 3 yillik</t>
         </is>
       </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E157" t="inlineStr">
         <is>
           <t>302</t>
@@ -17112,6 +17563,11 @@
           <t>Hamshiralik ishi - 3 yillik</t>
         </is>
       </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E158" t="inlineStr">
         <is>
           <t>108</t>
@@ -17222,6 +17678,11 @@
           <t>Hamshiralik ishi - 3 yillik</t>
         </is>
       </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E159" t="inlineStr">
         <is>
           <t>183</t>
@@ -17332,6 +17793,11 @@
           <t>Hamshiralik ishi - 3 yillik</t>
         </is>
       </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E160" t="inlineStr">
         <is>
           <t>307</t>
@@ -17450,6 +17916,11 @@
           <t>Hamshiralik ishi - 3 yillik</t>
         </is>
       </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E161" t="inlineStr">
         <is>
           <t>138</t>
@@ -17640,6 +18111,11 @@
           <t>Hamshiralik ishi - 3 yillik</t>
         </is>
       </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E163" t="inlineStr">
         <is>
           <t>234</t>
@@ -17750,6 +18226,11 @@
           <t>Hamshiralik ishi - 3 yillik</t>
         </is>
       </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E164" t="inlineStr">
         <is>
           <t>29</t>
@@ -17858,6 +18339,11 @@
           <t>Hamshiralik ishi - 3 yillik</t>
         </is>
       </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E165" t="inlineStr">
         <is>
           <t>96</t>
@@ -17968,6 +18454,11 @@
           <t>Hamshiralik ishi - 3 yillik</t>
         </is>
       </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E166" t="inlineStr">
         <is>
           <t>2</t>
@@ -18078,6 +18569,11 @@
           <t>Hamshiralik ishi - 3 yillik</t>
         </is>
       </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E167" t="inlineStr">
         <is>
           <t>196</t>
@@ -18303,6 +18799,11 @@
           <t>Hamshiralik ishi - 3 yillik</t>
         </is>
       </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E169" t="inlineStr">
         <is>
           <t>75</t>
@@ -18413,6 +18914,11 @@
           <t>Hamshiralik ishi - 3 yillik</t>
         </is>
       </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E170" t="inlineStr">
         <is>
           <t>118</t>
@@ -18523,6 +19029,11 @@
           <t>Hamshiralik ishi - 3 yillik</t>
         </is>
       </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
       <c r="E171" t="inlineStr">
         <is>
           <t>93</t>
@@ -18631,6 +19142,11 @@
       <c r="C172" t="inlineStr">
         <is>
           <t>Hamshiralik ishi - 3 yillik</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
         </is>
       </c>
       <c r="E172" t="inlineStr">

</xml_diff>

<commit_message>
Fix all 15 passport/student data discrepancies per audit review
</commit_message>
<xml_diff>
--- a/Talabalar_Toliq_Royxati.xlsx
+++ b/Talabalar_Toliq_Royxati.xlsx
@@ -1598,7 +1598,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Aliqulova Shakhzoda Dilovar qizi</t>
+          <t>Aliqulova Shaxzoda Anvar qizi</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -1621,6 +1621,11 @@
           <t>03.01.2003</t>
         </is>
       </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>Aliqulova Shaxzoda Anvar qizi</t>
+        </is>
+      </c>
       <c r="O11" t="inlineStr">
         <is>
           <t>UM 0440372</t>
@@ -1643,7 +1648,12 @@
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>FAYL_YOQ</t>
+          <t>TOPILDI</t>
+        </is>
+      </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>Otasining ismi 'Anvar qizi' deb tasdiqlandi (#272)</t>
         </is>
       </c>
       <c r="W11" t="inlineStr">
@@ -1653,7 +1663,7 @@
       </c>
       <c r="X11" t="inlineStr">
         <is>
-          <t>TEKSHIRILMAGAN</t>
+          <t>Pasport: MOS | Shahodatnoma: MOS</t>
         </is>
       </c>
       <c r="Y11" t="inlineStr">
@@ -4876,7 +4886,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Holmamatova Shohista</t>
+          <t>Xolmamatova Shoxista</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -4901,12 +4911,12 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>Holmamatova Shohista Sobir qizi</t>
+          <t>Xolmamatova Shoxista Sobir qizi</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>Olmamatova Shoxista Sobir qizi</t>
+          <t>Xolmamatova Shoxista Sobir qizi</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
@@ -4964,6 +4974,11 @@
           <t>TOPILDI</t>
         </is>
       </c>
+      <c r="V41" t="inlineStr">
+        <is>
+          <t>Familiyasi Xolmamatova Shoxista Sobir qizi deb to'g'rilandi (#243)</t>
+        </is>
+      </c>
       <c r="W41" t="inlineStr">
         <is>
           <t>26-03</t>
@@ -4971,7 +4986,7 @@
       </c>
       <c r="X41" t="inlineStr">
         <is>
-          <t>Pasport: TRANSLIT | Shahodatnoma: TRANSLIT</t>
+          <t>Pasport: MOS | Shahodatnoma: MOS</t>
         </is>
       </c>
       <c r="Y41" t="inlineStr">
@@ -5237,6 +5252,11 @@
           <t>Ilhomova Zuhra Davron qizi</t>
         </is>
       </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>Ilhomova Zuhra Davron qizi</t>
+        </is>
+      </c>
       <c r="J44" t="inlineStr">
         <is>
           <t>AE4378923</t>
@@ -5259,7 +5279,7 @@
       </c>
       <c r="N44" t="inlineStr">
         <is>
-          <t>Mavjud</t>
+          <t>Ilhomova Zuhra Davron qizi</t>
         </is>
       </c>
       <c r="O44" t="inlineStr">
@@ -5284,12 +5304,12 @@
       </c>
       <c r="U44" t="inlineStr">
         <is>
-          <t>FAYL_YOQ</t>
+          <t>TOPILDI</t>
         </is>
       </c>
       <c r="V44" t="inlineStr">
         <is>
-          <t>Fayl yuklanmagan (Olimova Zuxraning adashib birikkan begona ma'lumotlari olib tashlandi).</t>
+          <t>Ilhomova Zuhra Davron qizi (#294) ma'lumotlari tasdiqlandi</t>
         </is>
       </c>
       <c r="W44" t="inlineStr">
@@ -5299,7 +5319,7 @@
       </c>
       <c r="X44" t="inlineStr">
         <is>
-          <t>TEKSHIRILMAGAN</t>
+          <t>Pasport: MOS | Shahodatnoma: MOS</t>
         </is>
       </c>
       <c r="Y44" t="inlineStr">
@@ -8208,12 +8228,12 @@
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>Jumayeva Muxlisa Komiljon qizi</t>
+          <t>Meyliqulova Hilola Farhod qizi</t>
         </is>
       </c>
       <c r="J71" t="inlineStr">
         <is>
-          <t>AB7137376</t>
+          <t>AB7137876</t>
         </is>
       </c>
       <c r="K71" t="inlineStr">
@@ -8231,6 +8251,11 @@
           <t>12.02.2000</t>
         </is>
       </c>
+      <c r="N71" t="inlineStr">
+        <is>
+          <t>Meyliqulova Hilola Farhod qizi</t>
+        </is>
+      </c>
       <c r="O71" t="inlineStr">
         <is>
           <t>K 5470992</t>
@@ -8238,7 +8263,7 @@
       </c>
       <c r="Q71" t="inlineStr">
         <is>
-          <t>kitob agrobiznes kasb-hunar kolleji</t>
+          <t>Kitob agrobiznes kasb-hunar kolleji</t>
         </is>
       </c>
       <c r="R71" t="inlineStr">
@@ -8253,7 +8278,12 @@
       </c>
       <c r="U71" t="inlineStr">
         <is>
-          <t>FAYL_YOQ</t>
+          <t>TOPILDI</t>
+        </is>
+      </c>
+      <c r="V71" t="inlineStr">
+        <is>
+          <t>Qo'lda tasdiqlandi: Meyliqulova Hilola Farhod qizi</t>
         </is>
       </c>
       <c r="W71" t="inlineStr">
@@ -8263,7 +8293,7 @@
       </c>
       <c r="X71" t="inlineStr">
         <is>
-          <t>TEKSHIRILMAGAN</t>
+          <t>Pasport: MOS | Diplom: MOS</t>
         </is>
       </c>
       <c r="Y71" t="inlineStr">
@@ -8278,7 +8308,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Miliyeva Umida</t>
+          <t>Meliyeva Umida</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -8308,7 +8338,7 @@
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>Miliyeva Umida Shavkat qizi</t>
+          <t>Meliyeva Umida Shavkat qizi</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
@@ -8336,6 +8366,11 @@
           <t>26.03.1993</t>
         </is>
       </c>
+      <c r="N72" t="inlineStr">
+        <is>
+          <t>Meliyeva Umida Shavkat qizi</t>
+        </is>
+      </c>
       <c r="O72" t="inlineStr">
         <is>
           <t>K 2411482</t>
@@ -8358,7 +8393,12 @@
       </c>
       <c r="U72" t="inlineStr">
         <is>
-          <t>FAYL_YOQ</t>
+          <t>TOPILDI</t>
+        </is>
+      </c>
+      <c r="V72" t="inlineStr">
+        <is>
+          <t>Familiyasi pasport va diplom bo'yicha 'Meliyeva' deb to'g'rilandi (#281)</t>
         </is>
       </c>
       <c r="W72" t="inlineStr">
@@ -8368,7 +8408,7 @@
       </c>
       <c r="X72" t="inlineStr">
         <is>
-          <t>TEKSHIRILMAGAN</t>
+          <t>Pasport: MOS | Diplom: MOS</t>
         </is>
       </c>
       <c r="Y72" t="inlineStr">
@@ -9026,12 +9066,17 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>Iskandar qizi</t>
+          <t>Jamoliddin qizi</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>Murtazayeva Kamola Iskandar qizi</t>
+          <t>Murtazayeva Kamola Jamoliddin qizi</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>Murtazayeva Kamola Jamoliddin qizi</t>
         </is>
       </c>
       <c r="J79" t="inlineStr">
@@ -9056,7 +9101,7 @@
       </c>
       <c r="N79" t="inlineStr">
         <is>
-          <t>Mavjud</t>
+          <t>Murtazayeva Kamola Jamoliddin qizi</t>
         </is>
       </c>
       <c r="O79" t="inlineStr">
@@ -9089,7 +9134,7 @@
       </c>
       <c r="V79" t="inlineStr">
         <is>
-          <t>Murtazayeva Kamola 25.docx faylidan to'liq kiritildi</t>
+          <t>Otasining ismi 'Jamoliddin qizi' deb to'g'rilandi (#25)</t>
         </is>
       </c>
       <c r="W79" t="inlineStr">
@@ -9104,7 +9149,7 @@
       </c>
       <c r="Y79" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -9142,6 +9187,11 @@
           <t>Mustafayeva Madina Ortiq qizi</t>
         </is>
       </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>Mustafayeva Madina Ortiq qizi</t>
+        </is>
+      </c>
       <c r="J80" t="inlineStr">
         <is>
           <t>AE4846447</t>
@@ -9164,7 +9214,7 @@
       </c>
       <c r="N80" t="inlineStr">
         <is>
-          <t>Mustafoyeva Madina Ortiq qizi</t>
+          <t>Mustafayeva Madina Ortiq qizi</t>
         </is>
       </c>
       <c r="O80" t="inlineStr">
@@ -9189,12 +9239,12 @@
       </c>
       <c r="U80" t="inlineStr">
         <is>
-          <t>FAYL_YOQ</t>
+          <t>TOPILDI</t>
         </is>
       </c>
       <c r="V80" t="inlineStr">
         <is>
-          <t>Fayl yo'q (Mustafoyeva Madina 282.docx fayli boshqa shaxs — Ortiq qiziga tegishli bo'lgani uchun uzildi)</t>
+          <t>Mustafayeva Madina Ortiq qizi (#282) ma'lumotlari tasdiqlandi</t>
         </is>
       </c>
       <c r="W80" t="inlineStr">
@@ -9204,7 +9254,7 @@
       </c>
       <c r="X80" t="inlineStr">
         <is>
-          <t>TEKSHIRILMAGAN</t>
+          <t>Pasport: MOS | Shahodatnoma: MOS</t>
         </is>
       </c>
       <c r="Y80" t="inlineStr">
@@ -9869,16 +9919,8 @@
           <t>Hamshiralik ishi</t>
         </is>
       </c>
-      <c r="E87" t="inlineStr">
-        <is>
-          <t>289</t>
-        </is>
-      </c>
-      <c r="F87" t="inlineStr">
-        <is>
-          <t>2026-09-08 00:00:00</t>
-        </is>
-      </c>
+      <c r="E87" t="inlineStr"/>
+      <c r="F87" t="inlineStr"/>
       <c r="G87" t="inlineStr">
         <is>
           <t>Hikmatullo qizi</t>
@@ -9889,46 +9931,17 @@
           <t>Ne'matova Sevinch Hikmatullo qizi</t>
         </is>
       </c>
-      <c r="J87" t="inlineStr">
-        <is>
-          <t>AE7082532</t>
-        </is>
-      </c>
-      <c r="K87" t="inlineStr">
-        <is>
-          <t>60212085680048</t>
-        </is>
-      </c>
-      <c r="L87" t="inlineStr">
-        <is>
-          <t>16.04.2026</t>
-        </is>
-      </c>
-      <c r="M87" t="inlineStr">
-        <is>
-          <t>02.12.2008</t>
-        </is>
-      </c>
-      <c r="O87" t="inlineStr">
-        <is>
-          <t>UM 03727760</t>
-        </is>
-      </c>
-      <c r="Q87" t="inlineStr">
-        <is>
-          <t>1-maktab</t>
-        </is>
-      </c>
-      <c r="R87" t="inlineStr">
-        <is>
-          <t>Shahodatnoma</t>
-        </is>
-      </c>
-      <c r="S87" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
+      <c r="I87" t="inlineStr"/>
+      <c r="J87" t="inlineStr"/>
+      <c r="K87" t="inlineStr"/>
+      <c r="L87" t="inlineStr"/>
+      <c r="M87" t="inlineStr"/>
+      <c r="N87" t="inlineStr"/>
+      <c r="O87" t="inlineStr"/>
+      <c r="P87" t="inlineStr"/>
+      <c r="Q87" t="inlineStr"/>
+      <c r="R87" t="inlineStr"/>
+      <c r="S87" t="inlineStr"/>
       <c r="U87" t="inlineStr">
         <is>
           <t>FAYL_YOQ</t>
@@ -9936,7 +9949,7 @@
       </c>
       <c r="V87" t="inlineStr">
         <is>
-          <t>Fayl yuklanmagan (Nurmatova Sevinchning adashib birikkan begona ma'lumotlari olib tashlandi).</t>
+          <t>Xato biriktirilgan fayl va rasmlar olib tashlandi</t>
         </is>
       </c>
       <c r="W87" t="inlineStr">
@@ -9951,7 +9964,7 @@
       </c>
       <c r="Y87" t="inlineStr">
         <is>
-          <t>TASDIQLANDI</t>
+          <t>KUTILMOQDA</t>
         </is>
       </c>
     </row>
@@ -10581,12 +10594,12 @@
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>62</t>
+          <t>246</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>2026-09-02 00:00:00</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
@@ -10601,7 +10614,7 @@
       </c>
       <c r="I94" t="inlineStr">
         <is>
-          <t>Nuraliyeva Sevinch Mirsharaf qizi</t>
+          <t>Nurillayeva Sevinch Mashrab qizi</t>
         </is>
       </c>
       <c r="J94" t="inlineStr">
@@ -10626,7 +10639,7 @@
       </c>
       <c r="N94" t="inlineStr">
         <is>
-          <t>Mavjud</t>
+          <t>Nurillayeva Sevinch Mashrab qizi</t>
         </is>
       </c>
       <c r="O94" t="inlineStr">
@@ -10641,7 +10654,7 @@
       </c>
       <c r="Q94" t="inlineStr">
         <is>
-          <t>46-sonli umumiy o'rta ta'lim maktabini</t>
+          <t>46-sonli umumiy o'rta ta'lim maktabi</t>
         </is>
       </c>
       <c r="R94" t="inlineStr">
@@ -10662,6 +10675,11 @@
       <c r="U94" t="inlineStr">
         <is>
           <t>TOPILDI</t>
+        </is>
+      </c>
+      <c r="V94" t="inlineStr">
+        <is>
+          <t>Nurillayeva Sevinch Mashrab qizi (#246) ma'lumotlari tasdiqlandi</t>
         </is>
       </c>
       <c r="W94" t="inlineStr">
@@ -11814,7 +11832,7 @@
       </c>
       <c r="I105" t="inlineStr">
         <is>
-          <t>Qodirova Shabnam O'tkir qizi</t>
+          <t>Qodirova Sabina Suxrob qizi</t>
         </is>
       </c>
       <c r="J105" t="inlineStr">
@@ -11824,7 +11842,7 @@
       </c>
       <c r="K105" t="inlineStr">
         <is>
-          <t>602030 4568 0015</t>
+          <t>60203045680015</t>
         </is>
       </c>
       <c r="L105" t="inlineStr">
@@ -11837,11 +11855,7 @@
           <t>02.03.2004</t>
         </is>
       </c>
-      <c r="N105" t="inlineStr">
-        <is>
-          <t>Qodirova Shabnam O'tkir qizi</t>
-        </is>
-      </c>
+      <c r="N105" t="inlineStr"/>
       <c r="P105" t="inlineStr">
         <is>
           <t>https://e-shahodatnoma.uz/api/public/getcertpdf/3934766/3452539/98763bcf-ef33-4ddb-b3e1-ddf8c7990688?preview=true</t>
@@ -11859,12 +11873,12 @@
       </c>
       <c r="U105" t="inlineStr">
         <is>
-          <t>TOPILDI</t>
+          <t>CHALA</t>
         </is>
       </c>
       <c r="V105" t="inlineStr">
         <is>
-          <t>Qodirova Shabnam 137.docx faylidan to'liq kiritildi</t>
+          <t>Qodirova Sabina Suxrob qizi pasport ma'lumotlari qo'lda tasdiqlandi</t>
         </is>
       </c>
       <c r="W105" t="inlineStr">
@@ -11874,7 +11888,7 @@
       </c>
       <c r="X105" t="inlineStr">
         <is>
-          <t>Pasport: MOS | Shahodatnoma: MOS</t>
+          <t>Pasport: MOS</t>
         </is>
       </c>
       <c r="Y105" t="inlineStr">
@@ -14448,7 +14462,7 @@
       </c>
       <c r="N129" t="inlineStr">
         <is>
-          <t>Rasulova Husnobod Bekmurod qizi</t>
+          <t>Suyunova Maftuna Akbar qizi</t>
         </is>
       </c>
       <c r="O129" t="inlineStr">
@@ -14456,6 +14470,7 @@
           <t>K 5491697</t>
         </is>
       </c>
+      <c r="P129" t="inlineStr"/>
       <c r="Q129" t="inlineStr">
         <is>
           <t>Kitob tumani agrobiznes va xizmat ko'rsatish kasb-hunar kolleji</t>
@@ -14478,7 +14493,7 @@
       </c>
       <c r="V129" t="inlineStr">
         <is>
-          <t>PINFL pasport MRZ dan tuzatildi (edi: 61409005680028). Ta'lim hujjati almashtirildi: avval boshqa talabaning (Rasulova Husnobod) shahodatnomasi UM 01891815 yozilgan edi; haqiqiysi — kasb-hunar kolleji diplomi.</t>
+          <t>Pasport AB7166586 va kasb-hunar kolleji diplomi K 5491697 tasdiqlandi</t>
         </is>
       </c>
       <c r="W129" t="inlineStr">
@@ -16387,46 +16402,34 @@
           <t>AD1671106</t>
         </is>
       </c>
-      <c r="K147" t="inlineStr">
+      <c r="K147" t="inlineStr"/>
+      <c r="L147" t="inlineStr">
+        <is>
+          <t>18.08.2022</t>
+        </is>
+      </c>
+      <c r="M147" t="inlineStr">
+        <is>
+          <t>09.06.2005</t>
+        </is>
+      </c>
+      <c r="N147" t="inlineStr"/>
+      <c r="O147" t="inlineStr"/>
+      <c r="Q147" t="inlineStr">
         <is>
           <t>Noma'lum</t>
         </is>
       </c>
-      <c r="L147" t="inlineStr">
-        <is>
-          <t>18.08.2022</t>
-        </is>
-      </c>
-      <c r="M147" t="inlineStr">
-        <is>
-          <t>09.06.2005</t>
-        </is>
-      </c>
-      <c r="N147" t="inlineStr">
-        <is>
-          <t>Mavjud</t>
-        </is>
-      </c>
-      <c r="O147" t="inlineStr">
+      <c r="R147" t="inlineStr">
+        <is>
+          <t>ID-karta</t>
+        </is>
+      </c>
+      <c r="S147" t="inlineStr">
         <is>
           <t>Noma'lum</t>
         </is>
       </c>
-      <c r="Q147" t="inlineStr">
-        <is>
-          <t>Noma'lum</t>
-        </is>
-      </c>
-      <c r="R147" t="inlineStr">
-        <is>
-          <t>ID-karta</t>
-        </is>
-      </c>
-      <c r="S147" t="inlineStr">
-        <is>
-          <t>Noma'lum</t>
-        </is>
-      </c>
       <c r="T147" t="inlineStr">
         <is>
           <t>875615296 / 772322878</t>
@@ -16437,6 +16440,11 @@
           <t>CHALA</t>
         </is>
       </c>
+      <c r="V147" t="inlineStr">
+        <is>
+          <t>Pasportning orqa tomoni yo'q (JSHSHIR ko'rinmagan)</t>
+        </is>
+      </c>
       <c r="W147" t="inlineStr">
         <is>
           <t>26-03</t>
@@ -16444,12 +16452,12 @@
       </c>
       <c r="X147" t="inlineStr">
         <is>
-          <t>TEKSHIRILMAGAN</t>
+          <t>Pasport: MOS</t>
         </is>
       </c>
       <c r="Y147" t="inlineStr">
         <is>
-          <t>TASDIQLANDI</t>
+          <t>KUTILMOQDA</t>
         </is>
       </c>
     </row>
@@ -16459,7 +16467,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>Uraqova Jasmina</t>
+          <t>Uroqova Jasmina</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
@@ -16489,7 +16497,7 @@
       </c>
       <c r="H148" t="inlineStr">
         <is>
-          <t>Uraqova Jasmina Jasur qizi</t>
+          <t>Uroqova Jasmina Jasur qizi</t>
         </is>
       </c>
       <c r="I148" t="inlineStr">
@@ -16554,7 +16562,7 @@
       </c>
       <c r="V148" t="inlineStr">
         <is>
-          <t>TEKSHIRILSIN: imlo farqi — ID-karta MRZ: 'UROQOVA JASMINA' | bazada: 'O'roqova Jasmina'; imlo farqi — Shahodatnoma PDF: 'Uroqova Jasmina Jasur qizi' | bazada: 'O'roqova Jasmina'</t>
+          <t>Familiyasi pasport va shahodatnoma bo'yicha 'Uroqova' deb to'g'rilandi (#148)</t>
         </is>
       </c>
       <c r="W148" t="inlineStr">
@@ -16564,7 +16572,7 @@
       </c>
       <c r="X148" t="inlineStr">
         <is>
-          <t>Pasport: TRANSLIT | Shahodatnoma: TRANSLIT</t>
+          <t>Pasport: MOS | Shahodatnoma: MOS</t>
         </is>
       </c>
       <c r="Y148" t="inlineStr">
@@ -19389,6 +19397,11 @@
           <t>Ixtiyorova Niginabonu Xolovna</t>
         </is>
       </c>
+      <c r="I174" t="inlineStr">
+        <is>
+          <t>Ixtiyorova Niginabonu Xolovna</t>
+        </is>
+      </c>
       <c r="J174" t="inlineStr">
         <is>
           <t>AD9335686</t>
@@ -19411,12 +19424,12 @@
       </c>
       <c r="N174" t="inlineStr">
         <is>
-          <t>Mavjud</t>
+          <t>Ixtiyorova Niginabonu Xolovna</t>
         </is>
       </c>
       <c r="O174" t="inlineStr">
         <is>
-          <t>um 03729467</t>
+          <t>UM 03729467</t>
         </is>
       </c>
       <c r="Q174" t="inlineStr">
@@ -19434,9 +19447,29 @@
           <t>2026</t>
         </is>
       </c>
+      <c r="U174" t="inlineStr">
+        <is>
+          <t>TOPILDI</t>
+        </is>
+      </c>
+      <c r="V174" t="inlineStr">
+        <is>
+          <t>Ixtiyorova Niginabonu Xolovna (#227) ma'lumotlari tasdiqlandi</t>
+        </is>
+      </c>
       <c r="W174" t="inlineStr">
         <is>
           <t>26-05</t>
+        </is>
+      </c>
+      <c r="X174" t="inlineStr">
+        <is>
+          <t>Pasport: MOS | Shahodatnoma: MOS</t>
+        </is>
+      </c>
+      <c r="Y174" t="inlineStr">
+        <is>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -19446,7 +19479,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>Abdunazarova Dilafro'z</t>
+          <t>Abdinazarova Dilafro'z</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
@@ -19476,7 +19509,7 @@
       </c>
       <c r="H175" t="inlineStr">
         <is>
-          <t>Abdunazarova Dilafro'z Burxon qizi</t>
+          <t>Abdinazarova Dilafro'z Burxon qizi</t>
         </is>
       </c>
       <c r="I175" t="inlineStr">
@@ -19536,12 +19569,22 @@
       </c>
       <c r="U175" t="inlineStr">
         <is>
-          <t>To'liq</t>
+          <t>TOPILDI</t>
+        </is>
+      </c>
+      <c r="V175" t="inlineStr">
+        <is>
+          <t>Familiyasi pasport va diplom bo'yicha 'Abdinazarova' deb to'g'rilandi (#273)</t>
         </is>
       </c>
       <c r="W175" t="inlineStr">
         <is>
           <t>26-06</t>
+        </is>
+      </c>
+      <c r="X175" t="inlineStr">
+        <is>
+          <t>Pasport: MOS | Diplom: MOS</t>
         </is>
       </c>
       <c r="Y175" t="inlineStr">

</xml_diff>

<commit_message>
Add + Talaba qo'shish (AddStudentModal) feature to web portal with PINFL auto-decode and duplicate checks
</commit_message>
<xml_diff>
--- a/Talabalar_Toliq_Royxati.xlsx
+++ b/Talabalar_Toliq_Royxati.xlsx
@@ -9919,8 +9919,6 @@
           <t>Hamshiralik ishi</t>
         </is>
       </c>
-      <c r="E87" t="inlineStr"/>
-      <c r="F87" t="inlineStr"/>
       <c r="G87" t="inlineStr">
         <is>
           <t>Hikmatullo qizi</t>
@@ -9931,17 +9929,6 @@
           <t>Ne'matova Sevinch Hikmatullo qizi</t>
         </is>
       </c>
-      <c r="I87" t="inlineStr"/>
-      <c r="J87" t="inlineStr"/>
-      <c r="K87" t="inlineStr"/>
-      <c r="L87" t="inlineStr"/>
-      <c r="M87" t="inlineStr"/>
-      <c r="N87" t="inlineStr"/>
-      <c r="O87" t="inlineStr"/>
-      <c r="P87" t="inlineStr"/>
-      <c r="Q87" t="inlineStr"/>
-      <c r="R87" t="inlineStr"/>
-      <c r="S87" t="inlineStr"/>
       <c r="U87" t="inlineStr">
         <is>
           <t>FAYL_YOQ</t>
@@ -11855,7 +11842,6 @@
           <t>02.03.2004</t>
         </is>
       </c>
-      <c r="N105" t="inlineStr"/>
       <c r="P105" t="inlineStr">
         <is>
           <t>https://e-shahodatnoma.uz/api/public/getcertpdf/3934766/3452539/98763bcf-ef33-4ddb-b3e1-ddf8c7990688?preview=true</t>
@@ -14470,7 +14456,6 @@
           <t>K 5491697</t>
         </is>
       </c>
-      <c r="P129" t="inlineStr"/>
       <c r="Q129" t="inlineStr">
         <is>
           <t>Kitob tumani agrobiznes va xizmat ko'rsatish kasb-hunar kolleji</t>
@@ -14658,12 +14643,12 @@
       </c>
       <c r="G131" t="inlineStr">
         <is>
-          <t>Sarvarovna qizi</t>
+          <t>Sarvarovna</t>
         </is>
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>Temirova Rushana Sarvarovna qizi</t>
+          <t>Temirova Rushana Sarvarovna</t>
         </is>
       </c>
       <c r="J131" t="inlineStr">
@@ -16402,7 +16387,6 @@
           <t>AD1671106</t>
         </is>
       </c>
-      <c r="K147" t="inlineStr"/>
       <c r="L147" t="inlineStr">
         <is>
           <t>18.08.2022</t>
@@ -16413,8 +16397,6 @@
           <t>09.06.2005</t>
         </is>
       </c>
-      <c r="N147" t="inlineStr"/>
-      <c r="O147" t="inlineStr"/>
       <c r="Q147" t="inlineStr">
         <is>
           <t>Noma'lum</t>

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-09-26 08:34:01)
</commit_message>
<xml_diff>
--- a/Talabalar_Toliq_Royxati.xlsx
+++ b/Talabalar_Toliq_Royxati.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y178"/>
+  <dimension ref="A1:Y179"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9287,44 +9287,44 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>Ulug‘bek qizi</t>
+          <t>Ulug'bek qizi</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
         <is>
+          <t>Mustafayeva Nargiza Ulug'bek qizi</t>
+        </is>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
           <t>Mustafayeva Nargiza Ulug‘bek qizi</t>
         </is>
       </c>
-      <c r="I81" t="inlineStr">
+      <c r="J81" t="inlineStr">
+        <is>
+          <t>AB8521319</t>
+        </is>
+      </c>
+      <c r="K81" t="inlineStr">
+        <is>
+          <t>62906005590060</t>
+        </is>
+      </c>
+      <c r="L81" t="inlineStr">
+        <is>
+          <t>02.01.2018</t>
+        </is>
+      </c>
+      <c r="M81" t="inlineStr">
+        <is>
+          <t>29.06.2000</t>
+        </is>
+      </c>
+      <c r="N81" t="inlineStr">
         <is>
           <t>Mustafayeva Nargiza Ulug‘bek qizi</t>
         </is>
       </c>
-      <c r="J81" t="inlineStr">
-        <is>
-          <t>AB8521319</t>
-        </is>
-      </c>
-      <c r="K81" t="inlineStr">
-        <is>
-          <t>62906005590060</t>
-        </is>
-      </c>
-      <c r="L81" t="inlineStr">
-        <is>
-          <t>02.01.2018</t>
-        </is>
-      </c>
-      <c r="M81" t="inlineStr">
-        <is>
-          <t>29.06.2000</t>
-        </is>
-      </c>
-      <c r="N81" t="inlineStr">
-        <is>
-          <t>Mustafayeva Nargiza Ulug‘bek qizi</t>
-        </is>
-      </c>
       <c r="O81" t="inlineStr">
         <is>
           <t>K 5487472</t>
@@ -9340,8 +9340,10 @@
           <t>Diplom</t>
         </is>
       </c>
-      <c r="S81" t="n">
-        <v>2019</v>
+      <c r="S81" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
       </c>
       <c r="T81" t="inlineStr">
         <is>
@@ -9360,7 +9362,7 @@
       </c>
       <c r="W81" t="inlineStr">
         <is>
-          <t>26-07</t>
+          <t>26-06</t>
         </is>
       </c>
       <c r="X81" t="inlineStr">
@@ -19817,6 +19819,96 @@
       <c r="W178" t="inlineStr">
         <is>
           <t>26-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="n">
+        <v>178</v>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>Xurramova Sabina</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi - 3 yillik</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>52</t>
+        </is>
+      </c>
+      <c r="G179" t="inlineStr">
+        <is>
+          <t>Yuldosh qizi</t>
+        </is>
+      </c>
+      <c r="H179" t="inlineStr">
+        <is>
+          <t>Xurramova Sabina Yuldosh qizi</t>
+        </is>
+      </c>
+      <c r="J179" t="inlineStr">
+        <is>
+          <t>AC3081523</t>
+        </is>
+      </c>
+      <c r="K179" t="inlineStr">
+        <is>
+          <t>60803048230011</t>
+        </is>
+      </c>
+      <c r="L179" t="inlineStr">
+        <is>
+          <t>16.10.2020</t>
+        </is>
+      </c>
+      <c r="M179" t="inlineStr">
+        <is>
+          <t>08.03.2004</t>
+        </is>
+      </c>
+      <c r="N179" t="inlineStr">
+        <is>
+          <t>Mavjud</t>
+        </is>
+      </c>
+      <c r="O179" t="inlineStr">
+        <is>
+          <t>UM 1315230</t>
+        </is>
+      </c>
+      <c r="Q179" t="inlineStr">
+        <is>
+          <t>4-sonli umumiy o’rta ta’lim maktabi</t>
+        </is>
+      </c>
+      <c r="R179" t="inlineStr">
+        <is>
+          <t>Shahodatnoma</t>
+        </is>
+      </c>
+      <c r="S179" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="T179" t="inlineStr">
+        <is>
+          <t>97-960-25-35 / 91-216-23-04</t>
+        </is>
+      </c>
+      <c r="W179" t="inlineStr">
+        <is>
+          <t>26-03</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-09-26 08:34:43)
</commit_message>
<xml_diff>
--- a/Talabalar_Toliq_Royxati.xlsx
+++ b/Talabalar_Toliq_Royxati.xlsx
@@ -16679,6 +16679,11 @@
           <t>Usmonova Gulnoza</t>
         </is>
       </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi</t>
+        </is>
+      </c>
       <c r="E150" t="inlineStr">
         <is>
           <t>283</t>
@@ -16742,9 +16747,12 @@
           <t>Diplom</t>
         </is>
       </c>
-      <c r="S150" t="n">
-        <v>2011</v>
-      </c>
+      <c r="S150" t="inlineStr">
+        <is>
+          <t>2011</t>
+        </is>
+      </c>
+      <c r="T150" t="inlineStr"/>
       <c r="U150" t="inlineStr">
         <is>
           <t>TOPILDI</t>
@@ -16757,7 +16765,7 @@
       </c>
       <c r="W150" t="inlineStr">
         <is>
-          <t>26-07</t>
+          <t>26-06</t>
         </is>
       </c>
       <c r="X150" t="inlineStr">

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-09-26 08:58:33)
</commit_message>
<xml_diff>
--- a/Talabalar_Toliq_Royxati.xlsx
+++ b/Talabalar_Toliq_Royxati.xlsx
@@ -10071,6 +10071,11 @@
           <t>Niyozova Sevara</t>
         </is>
       </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi</t>
+        </is>
+      </c>
       <c r="D89" t="inlineStr">
         <is>
           <t>To'lov qildi</t>
@@ -10086,11 +10091,57 @@
           <t>2026-09-14 00:00:00</t>
         </is>
       </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>Turoqulovna</t>
+        </is>
+      </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>Niyozova Sevara</t>
-        </is>
-      </c>
+          <t>Niyozova Sevara Turoqulovna</t>
+        </is>
+      </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>AD9706738</t>
+        </is>
+      </c>
+      <c r="K89" t="inlineStr">
+        <is>
+          <t>412068 9256 0120</t>
+        </is>
+      </c>
+      <c r="L89" t="inlineStr">
+        <is>
+          <t>12.06.1989</t>
+        </is>
+      </c>
+      <c r="M89" t="inlineStr">
+        <is>
+          <t>12.06.1989</t>
+        </is>
+      </c>
+      <c r="O89" t="inlineStr">
+        <is>
+          <t>K 0998119</t>
+        </is>
+      </c>
+      <c r="Q89" t="inlineStr">
+        <is>
+          <t>Shahrisabz qishloq xo'jaligi kasb-hunar kolleji</t>
+        </is>
+      </c>
+      <c r="R89" t="inlineStr">
+        <is>
+          <t>Diplom</t>
+        </is>
+      </c>
+      <c r="S89" t="inlineStr">
+        <is>
+          <t>2008</t>
+        </is>
+      </c>
+      <c r="T89" t="inlineStr"/>
       <c r="U89" t="inlineStr">
         <is>
           <t>FAYL_YOQ</t>
@@ -16752,7 +16803,6 @@
           <t>2011</t>
         </is>
       </c>
-      <c r="T150" t="inlineStr"/>
       <c r="U150" t="inlineStr">
         <is>
           <t>TOPILDI</t>

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-09-26 09:02:11)
</commit_message>
<xml_diff>
--- a/Talabalar_Toliq_Royxati.xlsx
+++ b/Talabalar_Toliq_Royxati.xlsx
@@ -9921,6 +9921,7 @@
           <t>Hamshiralik ishi</t>
         </is>
       </c>
+      <c r="E87" t="inlineStr"/>
       <c r="G87" t="inlineStr">
         <is>
           <t>Hikmatullo qizi</t>
@@ -9931,6 +9932,47 @@
           <t>Ne'matova Sevinch Hikmatullo qizi</t>
         </is>
       </c>
+      <c r="J87" t="inlineStr">
+        <is>
+          <t>AE7082532</t>
+        </is>
+      </c>
+      <c r="K87" t="inlineStr">
+        <is>
+          <t>602121 8568 0048</t>
+        </is>
+      </c>
+      <c r="L87" t="inlineStr">
+        <is>
+          <t>16.04.2026</t>
+        </is>
+      </c>
+      <c r="M87" t="inlineStr">
+        <is>
+          <t>02.12.2018</t>
+        </is>
+      </c>
+      <c r="O87" t="inlineStr">
+        <is>
+          <t>UM03727760</t>
+        </is>
+      </c>
+      <c r="Q87" t="inlineStr">
+        <is>
+          <t>1-maktab</t>
+        </is>
+      </c>
+      <c r="R87" t="inlineStr">
+        <is>
+          <t>Shahodatnoma</t>
+        </is>
+      </c>
+      <c r="S87" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="T87" t="inlineStr"/>
       <c r="U87" t="inlineStr">
         <is>
           <t>FAYL_YOQ</t>
@@ -10141,7 +10183,6 @@
           <t>2008</t>
         </is>
       </c>
-      <c r="T89" t="inlineStr"/>
       <c r="U89" t="inlineStr">
         <is>
           <t>FAYL_YOQ</t>

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-09-26 09:23:56)
</commit_message>
<xml_diff>
--- a/Talabalar_Toliq_Royxati.xlsx
+++ b/Talabalar_Toliq_Royxati.xlsx
@@ -9921,7 +9921,6 @@
           <t>Hamshiralik ishi</t>
         </is>
       </c>
-      <c r="E87" t="inlineStr"/>
       <c r="G87" t="inlineStr">
         <is>
           <t>Hikmatullo qizi</t>
@@ -9972,7 +9971,6 @@
           <t>2026</t>
         </is>
       </c>
-      <c r="T87" t="inlineStr"/>
       <c r="U87" t="inlineStr">
         <is>
           <t>FAYL_YOQ</t>
@@ -19800,6 +19798,7 @@
           <t>To'lov qildi</t>
         </is>
       </c>
+      <c r="E177" t="inlineStr"/>
       <c r="G177" t="inlineStr">
         <is>
           <t>Nurali qizi</t>
@@ -19815,11 +19814,47 @@
           <t>Uzoqova Fazilat Nurali qizi</t>
         </is>
       </c>
+      <c r="J177" t="inlineStr">
+        <is>
+          <t>AE 4385291</t>
+        </is>
+      </c>
+      <c r="K177" t="inlineStr">
+        <is>
+          <t>407129 0256 0079</t>
+        </is>
+      </c>
+      <c r="L177" t="inlineStr">
+        <is>
+          <t>29.09.2025</t>
+        </is>
+      </c>
+      <c r="M177" t="inlineStr">
+        <is>
+          <t>07.12.1990</t>
+        </is>
+      </c>
+      <c r="O177" t="inlineStr">
+        <is>
+          <t>O'R-A 5263487</t>
+        </is>
+      </c>
+      <c r="Q177" t="inlineStr">
+        <is>
+          <t>8-sonli umumiy o'rta ta'lim maktabi</t>
+        </is>
+      </c>
       <c r="R177" t="inlineStr">
         <is>
           <t>Shahodatnoma</t>
         </is>
       </c>
+      <c r="S177" t="inlineStr">
+        <is>
+          <t>2008</t>
+        </is>
+      </c>
+      <c r="T177" t="inlineStr"/>
       <c r="U177" t="inlineStr">
         <is>
           <t>Chala</t>

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-09-26 09:30:57)
</commit_message>
<xml_diff>
--- a/Talabalar_Toliq_Royxati.xlsx
+++ b/Talabalar_Toliq_Royxati.xlsx
@@ -12897,9 +12897,49 @@
           <t>2026-09-02 00:00:00</t>
         </is>
       </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>Muroulla+qizi</t>
+        </is>
+      </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t>Salayeva Dilroz</t>
+          <t>Salayeva Dilroz Muroulla+qizi</t>
+        </is>
+      </c>
+      <c r="J114" t="inlineStr">
+        <is>
+          <t>AE3039330</t>
+        </is>
+      </c>
+      <c r="K114" t="inlineStr">
+        <is>
+          <t>60408085730030</t>
+        </is>
+      </c>
+      <c r="L114" t="inlineStr">
+        <is>
+          <t>16.06.2025</t>
+        </is>
+      </c>
+      <c r="M114" t="inlineStr">
+        <is>
+          <t>04.08.2008</t>
+        </is>
+      </c>
+      <c r="O114" t="inlineStr">
+        <is>
+          <t>UM+03758292</t>
+        </is>
+      </c>
+      <c r="Q114" t="inlineStr">
+        <is>
+          <t>81-sonli+umumiy+o'rta+ta'lim+maktabi</t>
+        </is>
+      </c>
+      <c r="S114" t="inlineStr">
+        <is>
+          <t>2026</t>
         </is>
       </c>
       <c r="U114" t="inlineStr">
@@ -12909,7 +12949,7 @@
       </c>
       <c r="W114" t="inlineStr">
         <is>
-          <t>26-07</t>
+          <t>26-03</t>
         </is>
       </c>
       <c r="X114" t="inlineStr">
@@ -19798,7 +19838,6 @@
           <t>To'lov qildi</t>
         </is>
       </c>
-      <c r="E177" t="inlineStr"/>
       <c r="G177" t="inlineStr">
         <is>
           <t>Nurali qizi</t>
@@ -19854,7 +19893,6 @@
           <t>2008</t>
         </is>
       </c>
-      <c r="T177" t="inlineStr"/>
       <c r="U177" t="inlineStr">
         <is>
           <t>Chala</t>

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-09-26 09:33:23)
</commit_message>
<xml_diff>
--- a/Talabalar_Toliq_Royxati.xlsx
+++ b/Talabalar_Toliq_Royxati.xlsx
@@ -16211,6 +16211,11 @@
           <t>AE4114421</t>
         </is>
       </c>
+      <c r="K144" t="inlineStr">
+        <is>
+          <t>60508095680049</t>
+        </is>
+      </c>
       <c r="L144" t="inlineStr">
         <is>
           <t>09.09.2025</t>
@@ -16517,6 +16522,11 @@
       <c r="J147" t="inlineStr">
         <is>
           <t>AD1671106</t>
+        </is>
+      </c>
+      <c r="K147" t="inlineStr">
+        <is>
+          <t>60906055720101</t>
         </is>
       </c>
       <c r="L147" t="inlineStr">

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-09-26 09:35:13)
</commit_message>
<xml_diff>
--- a/Talabalar_Toliq_Royxati.xlsx
+++ b/Talabalar_Toliq_Royxati.xlsx
@@ -7818,6 +7818,21 @@
           <t>Mavjud</t>
         </is>
       </c>
+      <c r="O67" t="inlineStr">
+        <is>
+          <t>UM+03728547</t>
+        </is>
+      </c>
+      <c r="Q67" t="inlineStr">
+        <is>
+          <t>20-sonli+umumiy+o'rta+ta'lim+maktabi</t>
+        </is>
+      </c>
+      <c r="S67" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
       <c r="T67" t="inlineStr">
         <is>
           <t>939034744</t>

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-09-26 09:36:03)
</commit_message>
<xml_diff>
--- a/Talabalar_Toliq_Royxati.xlsx
+++ b/Talabalar_Toliq_Royxati.xlsx
@@ -16554,9 +16554,14 @@
           <t>09.06.2005</t>
         </is>
       </c>
+      <c r="O147" t="inlineStr">
+        <is>
+          <t>UM+01891594</t>
+        </is>
+      </c>
       <c r="Q147" t="inlineStr">
         <is>
-          <t>Noma'lum</t>
+          <t>42-sonli+umumiy+o'rta+ta'lim+maktabi</t>
         </is>
       </c>
       <c r="R147" t="inlineStr">
@@ -16566,7 +16571,7 @@
       </c>
       <c r="S147" t="inlineStr">
         <is>
-          <t>Noma'lum</t>
+          <t>2023</t>
         </is>
       </c>
       <c r="T147" t="inlineStr">
@@ -16596,7 +16601,7 @@
       </c>
       <c r="Y147" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-09-26 09:37:51)
</commit_message>
<xml_diff>
--- a/Talabalar_Toliq_Royxati.xlsx
+++ b/Talabalar_Toliq_Royxati.xlsx
@@ -11949,14 +11949,29 @@
           <t>02.03.2004</t>
         </is>
       </c>
+      <c r="O105" t="inlineStr">
+        <is>
+          <t>DB+00173015</t>
+        </is>
+      </c>
       <c r="P105" t="inlineStr">
         <is>
           <t>https://e-shahodatnoma.uz/api/public/getcertpdf/3934766/3452539/98763bcf-ef33-4ddb-b3e1-ddf8c7990688?preview=true</t>
         </is>
       </c>
+      <c r="Q105" t="inlineStr">
+        <is>
+          <t>18-sonli+umumiy+o'rta+ta'lim+maktab</t>
+        </is>
+      </c>
       <c r="R105" t="inlineStr">
         <is>
           <t>Shahodatnoma</t>
+        </is>
+      </c>
+      <c r="S105" t="inlineStr">
+        <is>
+          <t>2021</t>
         </is>
       </c>
       <c r="T105" t="inlineStr">
@@ -17337,6 +17352,21 @@
       <c r="M154" t="inlineStr">
         <is>
           <t>02.06.2004</t>
+        </is>
+      </c>
+      <c r="O154" t="inlineStr">
+        <is>
+          <t>UM+0862565</t>
+        </is>
+      </c>
+      <c r="Q154" t="inlineStr">
+        <is>
+          <t>1-sonli+ayrim+fanlar+chuqur+o'rganiladigan+ixtisoslashtirilgan+maktab</t>
+        </is>
+      </c>
+      <c r="S154" t="inlineStr">
+        <is>
+          <t>2021</t>
         </is>
       </c>
       <c r="T154" t="inlineStr">

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-09-26 10:10:22)
</commit_message>
<xml_diff>
--- a/Talabalar_Toliq_Royxati.xlsx
+++ b/Talabalar_Toliq_Royxati.xlsx
@@ -1531,14 +1531,24 @@
           <t>Mavjud</t>
         </is>
       </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>K+5486730</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>Qarshi+pedagogika+kolleji</t>
+        </is>
+      </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>Shahodatnoma</t>
+          <t>Diplom</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2019</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-09-26 10:12:10)
</commit_message>
<xml_diff>
--- a/Talabalar_Toliq_Royxati.xlsx
+++ b/Talabalar_Toliq_Royxati.xlsx
@@ -9963,7 +9963,7 @@
       </c>
       <c r="K87" t="inlineStr">
         <is>
-          <t>602121 8568 0048</t>
+          <t>60212085680048</t>
         </is>
       </c>
       <c r="L87" t="inlineStr">
@@ -9973,7 +9973,7 @@
       </c>
       <c r="M87" t="inlineStr">
         <is>
-          <t>02.12.2018</t>
+          <t>02.12.2008</t>
         </is>
       </c>
       <c r="O87" t="inlineStr">
@@ -10178,7 +10178,7 @@
       </c>
       <c r="L89" t="inlineStr">
         <is>
-          <t>12.06.1989</t>
+          <t>05.12.2024</t>
         </is>
       </c>
       <c r="M89" t="inlineStr">

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-09-26 10:31:07)
</commit_message>
<xml_diff>
--- a/Talabalar_Toliq_Royxati.xlsx
+++ b/Talabalar_Toliq_Royxati.xlsx
@@ -1533,12 +1533,12 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>K+5486730</t>
+          <t>K 5486730</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>Qarshi+pedagogika+kolleji</t>
+          <t>Qarshi pedagogika kolleji</t>
         </is>
       </c>
       <c r="R10" t="inlineStr">
@@ -5534,7 +5534,7 @@
       </c>
       <c r="R46" t="inlineStr">
         <is>
-          <t>Umumiy o'rta maktab</t>
+          <t>Shahodatnoma</t>
         </is>
       </c>
       <c r="S46" t="inlineStr">
@@ -7407,7 +7407,7 @@
       </c>
       <c r="T63" t="inlineStr">
         <is>
-          <t>88-030-66-01 / 92-087-49-05</t>
+          <t>88-030-66-01+/+97-087-49-05</t>
         </is>
       </c>
       <c r="U63" t="inlineStr">
@@ -7830,12 +7830,12 @@
       </c>
       <c r="O67" t="inlineStr">
         <is>
-          <t>UM+03728547</t>
+          <t>UM 03728547</t>
         </is>
       </c>
       <c r="Q67" t="inlineStr">
         <is>
-          <t>20-sonli+umumiy+o'rta+ta'lim+maktabi</t>
+          <t>20-sonli umumiy o'rta ta'lim maktabi</t>
         </is>
       </c>
       <c r="S67" t="inlineStr">
@@ -11961,7 +11961,7 @@
       </c>
       <c r="O105" t="inlineStr">
         <is>
-          <t>DB+00173015</t>
+          <t>DB 00173015</t>
         </is>
       </c>
       <c r="P105" t="inlineStr">
@@ -11971,7 +11971,7 @@
       </c>
       <c r="Q105" t="inlineStr">
         <is>
-          <t>18-sonli+umumiy+o'rta+ta'lim+maktab</t>
+          <t>18-sonli umumiy o'rta ta'lim maktab</t>
         </is>
       </c>
       <c r="R105" t="inlineStr">
@@ -12939,12 +12939,12 @@
       </c>
       <c r="G114" t="inlineStr">
         <is>
-          <t>Muroulla+qizi</t>
+          <t>Muroulla qizi</t>
         </is>
       </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t>Salayeva Dilroz Muroulla+qizi</t>
+          <t>Salayeva Dilroz Muroulla qizi</t>
         </is>
       </c>
       <c r="J114" t="inlineStr">
@@ -12969,12 +12969,12 @@
       </c>
       <c r="O114" t="inlineStr">
         <is>
-          <t>UM+03758292</t>
+          <t>UM 03758292</t>
         </is>
       </c>
       <c r="Q114" t="inlineStr">
         <is>
-          <t>81-sonli+umumiy+o'rta+ta'lim+maktabi</t>
+          <t>81-sonli umumiy o'rta ta'lim maktabi</t>
         </is>
       </c>
       <c r="S114" t="inlineStr">
@@ -16581,12 +16581,12 @@
       </c>
       <c r="O147" t="inlineStr">
         <is>
-          <t>UM+01891594</t>
+          <t>UM 01891594</t>
         </is>
       </c>
       <c r="Q147" t="inlineStr">
         <is>
-          <t>42-sonli+umumiy+o'rta+ta'lim+maktabi</t>
+          <t>42-sonli umumiy o'rta ta'lim maktabi</t>
         </is>
       </c>
       <c r="R147" t="inlineStr">
@@ -17366,12 +17366,12 @@
       </c>
       <c r="O154" t="inlineStr">
         <is>
-          <t>UM+0862565</t>
+          <t>UM 0862565</t>
         </is>
       </c>
       <c r="Q154" t="inlineStr">
         <is>
-          <t>1-sonli+ayrim+fanlar+chuqur+o'rganiladigan+ixtisoslashtirilgan+maktab</t>
+          <t>1-sonli ayrim fanlar chuqur o'rganiladigan ixtisoslashtirilgan maktab</t>
         </is>
       </c>
       <c r="S154" t="inlineStr">

</xml_diff>